<commit_message>
Add validation-only scaled DQN monitor training
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -1348,7 +1348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1412,6 +1412,16 @@
           <t>elapsed_seconds</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>reward_scale</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>validation_only</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1456,6 +1466,8 @@
       <c r="L2" t="n">
         <v>37.50663828849792</v>
       </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1499,6 +1511,100 @@
       </c>
       <c r="L3" t="n">
         <v>51.22938394546509</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>smoke_ep10_rs100_val_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>47</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>32</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.14675124567906</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>125.0466907024384</v>
+      </c>
+      <c r="M4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>smoke_ep10_rs100_val_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>77</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>32</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.231519470803781</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>156.0144746303558</v>
+      </c>
+      <c r="M5" t="n">
+        <v>100</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add efficient validation scheduling for DQN runs
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -1348,7 +1348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1422,6 +1422,16 @@
           <t>validation_only</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>train_frequency</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>validate_every</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1468,6 +1478,8 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1514,6 +1526,8 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1560,6 +1574,8 @@
       <c r="N4" t="n">
         <v>1</v>
       </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1605,6 +1621,156 @@
       </c>
       <c r="N5" t="n">
         <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>full_ep2_rs100_val_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>47</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9151509841708554</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>259.417867898941</v>
+      </c>
+      <c r="M6" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>full_ep2_rs100_val_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>77</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>32</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.4129646565183226</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="n">
+        <v>259.775178194046</v>
+      </c>
+      <c r="M7" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>smoke_ep4_rs100_tf4_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>47</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>32</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="n">
+        <v>66.52740049362183</v>
+      </c>
+      <c r="M8" t="n">
+        <v>100</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add candidate-aware DQN controller oracle gate
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -10,7 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reference_sota" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pretrained_hrl" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dqn_runs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="final_comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oracle_runs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="final_comparison" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1348,7 +1349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1770,6 +1771,58 @@
         <v>4</v>
       </c>
       <c r="P8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>full_ep6_rs100_tf4_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>47</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>32</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.9501697377254155</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>880.5905005931854</v>
+      </c>
+      <c r="M9" t="n">
+        <v>100</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>4</v>
+      </c>
+      <c r="P9" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1784,6 +1837,427 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>reward_source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_cost</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_long</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>oracle_pass</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fixed_sharpe</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>fixed_switch_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>val_sharpe</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>val_return</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>max_dd</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>switch_count</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>transaction_cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.580805983196024</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2.936217593941671</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.2719376220703125</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0669978299520433</v>
+      </c>
+      <c r="M2" t="n">
+        <v>7</v>
+      </c>
+      <c r="N2" t="n">
+        <v>9.748408578336239</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.5400984129519202</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.580805983196024</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2.936217593941671</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.2719376220703125</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0669978299520433</v>
+      </c>
+      <c r="M3" t="n">
+        <v>7</v>
+      </c>
+      <c r="N3" t="n">
+        <v>9.748408578336239</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5400984129519202</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3.580805983196024</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3.289065786487285</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.3111237792968751</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.06702177854096704</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N4" t="n">
+        <v>7.034495489671826</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.3988379593356512</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2.666521915451586</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2.133127669708426</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.31632666015625</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.1519295253163833</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5.925663992762566</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.3444067824748345</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2.666521915451586</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2.133127669708426</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.31632666015625</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1519295253163833</v>
+      </c>
+      <c r="M6" t="n">
+        <v>3</v>
+      </c>
+      <c r="N6" t="n">
+        <v>5.925663992762566</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.3444067824748345</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>oracle_smoke_candidate_v2_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>outer_value</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2.666521915451586</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2.133127669708426</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.31632666015625</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.1519295253163833</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="n">
+        <v>5.925663992762566</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.3444067824748345</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Add policy gradient monitor controller
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -11,7 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pretrained_hrl" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dqn_runs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="oracle_runs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="final_comparison" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conditional_critic_runs" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="final_comparison" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pg_controller_runs" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -480,7 +482,6 @@
           <t>nas100</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>return</t>
@@ -763,12 +764,6 @@
           <t>DeepAries</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -896,7 +891,6 @@
           <t>sh</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>return</t>
@@ -1179,12 +1173,6 @@
           <t>DeepAries</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1227,12 +1215,6 @@
           <t>outer_only</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1245,12 +1227,6 @@
           <t>outer&amp;inner</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1263,12 +1239,6 @@
           <t>outer&amp;inner&amp;monitor</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1477,10 +1447,6 @@
       <c r="L2" t="n">
         <v>37.50663828849792</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1525,10 +1491,6 @@
       <c r="L3" t="n">
         <v>51.22938394546509</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1564,8 +1526,6 @@
       <c r="I4" t="n">
         <v>3.14675124567906</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>125.0466907024384</v>
       </c>
@@ -1575,8 +1535,6 @@
       <c r="N4" t="n">
         <v>1</v>
       </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1612,8 +1570,6 @@
       <c r="I5" t="n">
         <v>3.231519470803781</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>156.0144746303558</v>
       </c>
@@ -1623,8 +1579,6 @@
       <c r="N5" t="n">
         <v>1</v>
       </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1660,8 +1614,6 @@
       <c r="I6" t="n">
         <v>0.9151509841708554</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>259.417867898941</v>
       </c>
@@ -1671,8 +1623,6 @@
       <c r="N6" t="n">
         <v>1</v>
       </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1708,8 +1658,6 @@
       <c r="I7" t="n">
         <v>0.4129646565183226</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>259.775178194046</v>
       </c>
@@ -1719,8 +1667,6 @@
       <c r="N7" t="n">
         <v>1</v>
       </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1756,8 +1702,6 @@
       <c r="I8" t="n">
         <v>3.104039241616181</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>66.52740049362183</v>
       </c>
@@ -1808,8 +1752,6 @@
       <c r="I9" t="n">
         <v>0.9501697377254155</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>880.5905005931854</v>
       </c>
@@ -2258,6 +2200,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>episodes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_long</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>val_sharpe</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>val_return</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>utility_mse</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>switch_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>transaction_cost</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>elapsed_seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>conditional_smoke_candidate_v2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.217969144935847</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2775389404296875</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.0009025801970340983</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3.884147141128778</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.234054214641219</v>
+      </c>
+      <c r="L2" t="n">
+        <v>61.40583491325378</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>conditional_smoke_candidate_v2_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.857584227498245</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.4336228027343749</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.001429076804140942</v>
+      </c>
+      <c r="I3" t="n">
+        <v>88</v>
+      </c>
+      <c r="J3" t="n">
+        <v>88.3914754986763</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5.429019254923332</v>
+      </c>
+      <c r="L3" t="n">
+        <v>70.22009015083313</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2596,4 +2702,417 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>run_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mode</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>episodes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>lr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_min</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>lambda_max</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>val_sharpe</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>val_return</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>val_maxdd</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>switch_count</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>avg_hold_days</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>early_violation_count</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>long_violation_count</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>early_violation_rate</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>long_violation_rate</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>transaction_cost</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>test_status</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>elapsed_seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>47</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.183361203481455</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.2965123291015626</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.06573211836791722</v>
+      </c>
+      <c r="L2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5.809523809523809</v>
+      </c>
+      <c r="N2" t="n">
+        <v>21</v>
+      </c>
+      <c r="O2" t="n">
+        <v>41</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1721311475409836</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.3360655737704918</v>
+      </c>
+      <c r="R2" t="n">
+        <v>22.40794236212969</v>
+      </c>
+      <c r="S2" t="n">
+        <v>1.18928631694871</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>50.60620379447937</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>77</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.502546338049612</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.332495361328125</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.1375882134941958</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>116</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>85</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.7327586206896551</v>
+      </c>
+      <c r="R3" t="n">
+        <v>2.521827651187778</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.1559635098092258</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>54.14467310905457</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_direct_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>47</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>122</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>61</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>41.23095703125</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_direct_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>77</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.502546338049612</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.332495361328125</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1375882134941958</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>116</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>85</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.7327586206896551</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2.521827651187778</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.1559635098092258</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>55.41980743408203</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix PG controller holding constraints
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2710,7 +2710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:AD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2819,6 +2819,51 @@
           <t>elapsed_seconds</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>val_objective</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>val_penalty</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>constraint_loss_scale</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>grad_clip</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch_pre_min</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch_post_max</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_hold_post_max</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>constraint_logit_bias</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2892,6 +2937,15 @@
       <c r="U2" t="n">
         <v>50.60620379447937</v>
       </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2965,6 +3019,15 @@
       <c r="U3" t="n">
         <v>54.14467310905457</v>
       </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3038,6 +3101,15 @@
       <c r="U4" t="n">
         <v>41.23095703125</v>
       </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3110,6 +3182,849 @@
       </c>
       <c r="U5" t="n">
         <v>55.41980743408203</v>
+      </c>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_penalty100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>47</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" t="n">
+        <v>100</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>122</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>62</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S6" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>57.03308749198914</v>
+      </c>
+      <c r="V6" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_penalty100_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>77</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" t="n">
+        <v>100</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.502546338049612</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.332495361328125</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.1375882134941958</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>116</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>86</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0.7413793103448276</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2.521827651187778</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0.1559635098092258</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>56.40351176261902</v>
+      </c>
+      <c r="V7" t="n">
+        <v>-8597.49745366195</v>
+      </c>
+      <c r="W7" t="n">
+        <v>8600</v>
+      </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_penalty100_surrogate_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>47</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G8" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" t="n">
+        <v>100</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>122</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>62</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>39.24876737594604</v>
+      </c>
+      <c r="V8" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W8" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_penalty100_len80_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>47</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" t="n">
+        <v>100</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>122</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>62</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>52.62102079391479</v>
+      </c>
+      <c r="V9" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W9" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep5_penalty100_grad10_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>47</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" t="n">
+        <v>100</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>122</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>62</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R10" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>126.8963077068329</v>
+      </c>
+      <c r="V10" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W10" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_penalty100_probdiag_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>47</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G11" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" t="n">
+        <v>100</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>122</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>62</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>53.54163098335266</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W11" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0.4689881181130644</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.475618851184845</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.4669963414630582</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0.5330036580562592</v>
+      </c>
+      <c r="AD11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep5_lmin10_lmax1000_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>47</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>122</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>62</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R12" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>127.1960549354553</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-61996.89596075838</v>
+      </c>
+      <c r="W12" t="n">
+        <v>62000</v>
+      </c>
+      <c r="X12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0.4689958330060615</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.4756315946578979</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.4670004806210918</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0.5329995193789082</v>
+      </c>
+      <c r="AD12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_barrier10_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>47</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" t="n">
+        <v>100</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L13" t="n">
+        <v>24</v>
+      </c>
+      <c r="M13" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S13" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>52.90873861312866</v>
+      </c>
+      <c r="V13" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0.1079778584206325</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>5.518306318904529e-05</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pg_smoke_ep2_barrier10_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>77</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G14" t="n">
+        <v>100</v>
+      </c>
+      <c r="H14" t="n">
+        <v>100</v>
+      </c>
+      <c r="I14" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L14" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" t="n">
+        <v>29</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>58.7101731300354</v>
+      </c>
+      <c r="V14" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0.3615283100245882</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>3.184991060954737e-05</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>0.9999324878056844</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>6.746305492318545e-05</v>
+      </c>
+      <c r="AD14" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add controller decision diagnostics and late-hold search
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2710,7 +2710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD14"/>
+  <dimension ref="A1:AT30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2862,6 +2862,86 @@
       <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>constraint_logit_bias</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>hidden_dim</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>fusion_hidden</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>schedule_penalty</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_mean</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_std</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_min</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_max</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>scheduled_switch_count</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>scheduled_switch_rate</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>near_max_switch_count</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>near_max_switch_rate</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>min_hold_switch_count</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>min_hold_switch_rate</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>late_hold_start</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>late_hold_logit_bias</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>late_hold_loss_scale</t>
         </is>
       </c>
     </row>
@@ -2946,6 +3026,22 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3028,6 +3124,22 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3110,6 +3222,22 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3192,6 +3320,22 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3278,6 +3422,22 @@
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3364,6 +3524,22 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3452,6 +3628,22 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3540,6 +3732,22 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3630,6 +3838,22 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3728,6 +3952,22 @@
         <v>0.5330036580562592</v>
       </c>
       <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3826,6 +4066,22 @@
         <v>0.5329995193789082</v>
       </c>
       <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3926,6 +4182,22 @@
       <c r="AD13" t="n">
         <v>10</v>
       </c>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4024,6 +4296,2176 @@
         <v>6.746305492318545e-05</v>
       </c>
       <c r="AD14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias6_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>47</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" t="n">
+        <v>100</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.014349942670689</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.2495347900390625</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.07461822112307778</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>5.159690571948886</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0.3088942771428265</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>170.0867764949799</v>
+      </c>
+      <c r="V15" t="n">
+        <v>3.014349942670689</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0.4409939360892645</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>0.002223283029161394</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>0.9971909821033478</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>0.002809021505527198</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias8_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>47</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G16" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" t="n">
+        <v>100</v>
+      </c>
+      <c r="I16" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L16" t="n">
+        <v>24</v>
+      </c>
+      <c r="M16" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S16" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>75.20408058166504</v>
+      </c>
+      <c r="V16" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="W16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0.1082632838696867</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>0.0004076494238985588</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD16" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE16" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias10_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>47</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="n">
+        <v>100</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L17" t="n">
+        <v>24</v>
+      </c>
+      <c r="M17" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S17" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>73.27445435523987</v>
+      </c>
+      <c r="V17" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0.1079778584206325</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>5.518306318904529e-05</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF17" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias12_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>47</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G18" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" t="n">
+        <v>100</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L18" t="n">
+        <v>24</v>
+      </c>
+      <c r="M18" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S18" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>71.03069996833801</v>
+      </c>
+      <c r="V18" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="W18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0.1079359360820289</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>7.468027039364216e-06</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>12</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF18" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias6_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>77</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G19" t="n">
+        <v>100</v>
+      </c>
+      <c r="H19" t="n">
+        <v>100</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L19" t="n">
+        <v>3</v>
+      </c>
+      <c r="M19" t="n">
+        <v>29</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S19" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>79.38818860054016</v>
+      </c>
+      <c r="V19" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="W19" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0.3614320692010143</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>0.001732045202516019</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>0.9963225523630778</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0.003677472627411286</v>
+      </c>
+      <c r="AD19" t="n">
+        <v>6</v>
+      </c>
+      <c r="AE19" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias8_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>77</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G20" t="n">
+        <v>100</v>
+      </c>
+      <c r="H20" t="n">
+        <v>100</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3</v>
+      </c>
+      <c r="M20" t="n">
+        <v>29</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>79.62127423286438</v>
+      </c>
+      <c r="V20" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="W20" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0.3615334553061734</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>0.0002352192968828604</v>
+      </c>
+      <c r="AB20" t="n">
+        <v>0.999501625696818</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>0.0004983854984554151</v>
+      </c>
+      <c r="AD20" t="n">
+        <v>8</v>
+      </c>
+      <c r="AE20" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias10_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>77</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>100</v>
+      </c>
+      <c r="H21" t="n">
+        <v>100</v>
+      </c>
+      <c r="I21" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L21" t="n">
+        <v>3</v>
+      </c>
+      <c r="M21" t="n">
+        <v>29</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>82.72471523284912</v>
+      </c>
+      <c r="V21" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="W21" t="n">
+        <v>0</v>
+      </c>
+      <c r="X21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>0.3615283100245882</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>3.184991060954737e-05</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0.9999324878056844</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>6.746305492318545e-05</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE21" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>pg_smoke_bias_grid_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias12_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>77</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H22" t="n">
+        <v>100</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L22" t="n">
+        <v>3</v>
+      </c>
+      <c r="M22" t="n">
+        <v>29</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>78.1385703086853</v>
+      </c>
+      <c r="V22" t="n">
+        <v>2.217076848903197</v>
+      </c>
+      <c r="W22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0.3615306014385051</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>4.310641115272815e-06</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>0.9999908606211344</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>9.129349564318545e-06</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>12</v>
+      </c>
+      <c r="AE22" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>30</v>
+      </c>
+      <c r="AK22" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pg_smoke_lowbar_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias4_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>47</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G23" t="n">
+        <v>100</v>
+      </c>
+      <c r="H23" t="n">
+        <v>100</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.014349942670689</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.2495347900390625</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.07461822112307778</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2</v>
+      </c>
+      <c r="M23" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" t="n">
+        <v>5.159690571948886</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0.3088942771428265</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>72.38540005683899</v>
+      </c>
+      <c r="V23" t="n">
+        <v>2.514349942670689</v>
+      </c>
+      <c r="W23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0.4416348774474664</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>0.01618867106735706</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>0.979583203792572</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>0.02041676919907331</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE23" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AK23" t="n">
+        <v>60</v>
+      </c>
+      <c r="AL23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>pg_smoke_lowbar_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias5_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>47</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" t="n">
+        <v>100</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3.014349942670689</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.2495347900390625</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.07461822112307778</v>
+      </c>
+      <c r="L24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>5.159690571948886</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.3088942771428265</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>72.19550275802612</v>
+      </c>
+      <c r="V24" t="n">
+        <v>2.514349942670689</v>
+      </c>
+      <c r="W24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0.4409929131516485</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>0.006017576018348336</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>0.9923891723155975</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0.007610834203660488</v>
+      </c>
+      <c r="AD24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>60</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>60</v>
+      </c>
+      <c r="AK24" t="n">
+        <v>60</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias4_late0_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>47</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G25" t="n">
+        <v>100</v>
+      </c>
+      <c r="H25" t="n">
+        <v>100</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3.014349942670689</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.2495347900390625</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.07461822112307778</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2</v>
+      </c>
+      <c r="M25" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="n">
+        <v>5.159690571948886</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0.3088942771428265</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>71.53263783454895</v>
+      </c>
+      <c r="V25" t="n">
+        <v>2.514349942670689</v>
+      </c>
+      <c r="W25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0.4416348774474664</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>0.01618867106735706</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>0.979583203792572</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0.02041676919907331</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>60</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>60</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>60</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias4_late1_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>47</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G26" t="n">
+        <v>100</v>
+      </c>
+      <c r="H26" t="n">
+        <v>100</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3.455114537507225</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.2821976318359376</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.05408010690715014</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="n">
+        <v>5.38091211207211</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0.320458160713315</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>72.57036352157593</v>
+      </c>
+      <c r="V26" t="n">
+        <v>3.455114537507225</v>
+      </c>
+      <c r="W26" t="n">
+        <v>0</v>
+      </c>
+      <c r="X26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0.3586298835799709</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>0.01167399400415329</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK26" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_nas100_ep3_h32_f64_lr0p001_ent0p01_bias4_late2_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>47</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H27" t="n">
+        <v>100</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3.181063946730663</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.2854052734375001</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.07779889044782343</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="n">
+        <v>4.815671060234308</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0.2866742147598416</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>72.19550156593323</v>
+      </c>
+      <c r="V27" t="n">
+        <v>3.181063946730663</v>
+      </c>
+      <c r="W27" t="n">
+        <v>0</v>
+      </c>
+      <c r="X27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0.4250405621791228</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>0.01622377722882307</v>
+      </c>
+      <c r="AB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD27" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>43</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ27" t="n">
+        <v>43</v>
+      </c>
+      <c r="AK27" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias4_late0_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>77</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H28" t="n">
+        <v>100</v>
+      </c>
+      <c r="I28" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L28" t="n">
+        <v>3</v>
+      </c>
+      <c r="M28" t="n">
+        <v>29</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>76.81934809684753</v>
+      </c>
+      <c r="V28" t="n">
+        <v>2.217076848903197</v>
+      </c>
+      <c r="W28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0.362376103731643</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>0.01264633747803814</v>
+      </c>
+      <c r="AB28" t="n">
+        <v>0.9734256267547607</v>
+      </c>
+      <c r="AC28" t="n">
+        <v>0.02657439062992732</v>
+      </c>
+      <c r="AD28" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ28" t="n">
+        <v>30</v>
+      </c>
+      <c r="AK28" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias4_late1_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>77</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G29" t="n">
+        <v>100</v>
+      </c>
+      <c r="H29" t="n">
+        <v>100</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3.04661759413849</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.4819249267578125</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.09709203938712244</v>
+      </c>
+      <c r="L29" t="n">
+        <v>4</v>
+      </c>
+      <c r="M29" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>8.979459723457694</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0.5831022770726122</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>78.05838751792908</v>
+      </c>
+      <c r="V29" t="n">
+        <v>3.04661759413849</v>
+      </c>
+      <c r="W29" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0.3441333241102382</v>
+      </c>
+      <c r="AA29" t="n">
+        <v>0.0124391953771313</v>
+      </c>
+      <c r="AB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>24</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ29" t="n">
+        <v>24</v>
+      </c>
+      <c r="AK29" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>pg_smoke_late_ep3_sh_ep3_h32_f64_lr0p001_ent0p01_bias4_late2_lm100_lx100</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>77</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G30" t="n">
+        <v>100</v>
+      </c>
+      <c r="H30" t="n">
+        <v>100</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3.04661759413849</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.4819249267578125</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.09709203938712244</v>
+      </c>
+      <c r="L30" t="n">
+        <v>4</v>
+      </c>
+      <c r="M30" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="n">
+        <v>8.979459723457694</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0.5831022770726122</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>76.72955012321472</v>
+      </c>
+      <c r="V30" t="n">
+        <v>3.04661759413849</v>
+      </c>
+      <c r="W30" t="n">
+        <v>0</v>
+      </c>
+      <c r="X30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0.2858047790439992</v>
+      </c>
+      <c r="AA30" t="n">
+        <v>0.008753817351091476</v>
+      </c>
+      <c r="AB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>24</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ30" t="n">
+        <v>24</v>
+      </c>
+      <c r="AK30" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT30" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add reward-to-go PG objective and eval mode
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2364,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:AJ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2458,6 +2458,96 @@
           <t>dqn_loss</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_mean</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_std</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_min</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>switch_age_max</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>scheduled_switch_count</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>scheduled_switch_rate</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>near_max_switch_count</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>near_max_switch_rate</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>min_hold_switch_count</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>min_hold_switch_rate</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>early_violation_count</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>long_violation_count</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>early_violation_rate</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>long_violation_rate</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch_pre_min</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_switch_post_max</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>avg_p_hold_post_max</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2518,6 +2608,24 @@
         <v>0.4382022471910113</v>
       </c>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2578,6 +2686,24 @@
         <v>0.8764044943820225</v>
       </c>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2638,6 +2764,24 @@
         <v>0.4347826086956522</v>
       </c>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2698,6 +2842,132 @@
         <v>0.3739130434782609</v>
       </c>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pg_eval_test_sh_full_late1_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8371134033203125</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.1501278857468478</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2331748675184311</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.6438424556907127</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.2304033253803784</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.6515872936431154</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1837.113403320312</v>
+      </c>
+      <c r="K6" t="n">
+        <v>43</v>
+      </c>
+      <c r="L6" t="n">
+        <v>28.31818181818182</v>
+      </c>
+      <c r="M6" t="n">
+        <v>96.19963174127042</v>
+      </c>
+      <c r="N6" t="n">
+        <v>7.212756619235734</v>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>28.53488372093023</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.4987816416169121</v>
+      </c>
+      <c r="U6" t="n">
+        <v>28</v>
+      </c>
+      <c r="V6" t="n">
+        <v>29</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>43</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>0.2864533786670893</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0.007378935629743977</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2710,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT30"/>
+  <dimension ref="A1:AW37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2942,6 +3212,21 @@
       <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>late_hold_loss_scale</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>near_max_penalty</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>pg_objective</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>reward_gamma</t>
         </is>
       </c>
     </row>
@@ -3042,6 +3327,9 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3140,6 +3428,9 @@
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
       <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3238,6 +3529,9 @@
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
       <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3336,6 +3630,9 @@
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3438,6 +3735,9 @@
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3540,6 +3840,9 @@
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3644,6 +3947,9 @@
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3748,6 +4054,9 @@
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3854,6 +4163,9 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3968,6 +4280,9 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4082,6 +4397,9 @@
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4198,6 +4516,9 @@
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4314,6 +4635,9 @@
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4434,6 +4758,9 @@
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4554,6 +4881,9 @@
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4674,6 +5004,9 @@
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4794,6 +5127,9 @@
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4914,6 +5250,9 @@
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5034,6 +5373,9 @@
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5154,6 +5496,9 @@
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5296,6 +5641,9 @@
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
       <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5438,6 +5786,9 @@
       <c r="AR23" t="inlineStr"/>
       <c r="AS23" t="inlineStr"/>
       <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5580,6 +5931,9 @@
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="inlineStr"/>
       <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5728,6 +6082,9 @@
       <c r="AT25" t="n">
         <v>10</v>
       </c>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5876,6 +6233,9 @@
       <c r="AT26" t="n">
         <v>10</v>
       </c>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6024,6 +6384,9 @@
       <c r="AT27" t="n">
         <v>10</v>
       </c>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6172,6 +6535,9 @@
       <c r="AT28" t="n">
         <v>10</v>
       </c>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6320,6 +6686,9 @@
       <c r="AT29" t="n">
         <v>10</v>
       </c>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6467,6 +6836,1084 @@
       </c>
       <c r="AT30" t="n">
         <v>10</v>
+      </c>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>pg_full_ep8_nas100_late1_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>47</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G31" t="n">
+        <v>100</v>
+      </c>
+      <c r="H31" t="n">
+        <v>100</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.8977244329178085</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.5754620361328124</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.3018072524298372</v>
+      </c>
+      <c r="L31" t="n">
+        <v>11</v>
+      </c>
+      <c r="M31" t="n">
+        <v>48.16666666666666</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="n">
+        <v>24.96300726011395</v>
+      </c>
+      <c r="S31" t="n">
+        <v>1.590225962776458</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U31" t="n">
+        <v>1408.048740386963</v>
+      </c>
+      <c r="V31" t="n">
+        <v>0.8977244329178085</v>
+      </c>
+      <c r="W31" t="n">
+        <v>0</v>
+      </c>
+      <c r="X31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0.3696464037886824</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>0.01172476358787746</v>
+      </c>
+      <c r="AB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ31" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK31" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>pg_full_ep8_sh_late1_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>77</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G32" t="n">
+        <v>100</v>
+      </c>
+      <c r="H32" t="n">
+        <v>100</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1.114545684592665</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.5868944091796875</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.1738595037286902</v>
+      </c>
+      <c r="L32" t="n">
+        <v>17</v>
+      </c>
+      <c r="M32" t="n">
+        <v>26.94444444444444</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" t="n">
+        <v>38.59381351433694</v>
+      </c>
+      <c r="S32" t="n">
+        <v>2.303586967376759</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>1527.078641891479</v>
+      </c>
+      <c r="V32" t="n">
+        <v>1.114545684592665</v>
+      </c>
+      <c r="W32" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0.286828490163286</v>
+      </c>
+      <c r="AA32" t="n">
+        <v>0.007550295881009189</v>
+      </c>
+      <c r="AB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>28.47058823529412</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>0.4991341984846218</v>
+      </c>
+      <c r="AJ32" t="n">
+        <v>28</v>
+      </c>
+      <c r="AK32" t="n">
+        <v>29</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>17</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>pg_full_ep6_sh_late_start06_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>77</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G33" t="n">
+        <v>100</v>
+      </c>
+      <c r="H33" t="n">
+        <v>100</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.9211123408136285</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.4601424560546874</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.2455060497685057</v>
+      </c>
+      <c r="L33" t="n">
+        <v>17</v>
+      </c>
+      <c r="M33" t="n">
+        <v>26.94444444444444</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>36.68699019774795</v>
+      </c>
+      <c r="S33" t="n">
+        <v>2.016029110440286</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>1086.942515611649</v>
+      </c>
+      <c r="V33" t="n">
+        <v>0.4211123408136285</v>
+      </c>
+      <c r="W33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X33" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0.292689108431877</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>0.007533983914309168</v>
+      </c>
+      <c r="AB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD33" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>28</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0.4850712500726659</v>
+      </c>
+      <c r="AJ33" t="n">
+        <v>27</v>
+      </c>
+      <c r="AK33" t="n">
+        <v>29</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>17</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>pg_eval_test_sh_full_late1_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>77</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>eval_test</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G34" t="n">
+        <v>100</v>
+      </c>
+      <c r="H34" t="n">
+        <v>100</v>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="n">
+        <v>43</v>
+      </c>
+      <c r="M34" t="n">
+        <v>28.31818181818182</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="n">
+        <v>96.19963174127042</v>
+      </c>
+      <c r="S34" t="n">
+        <v>7.212756619235734</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U34" t="n">
+        <v>224.2061791419983</v>
+      </c>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0.2864533786670893</v>
+      </c>
+      <c r="AA34" t="n">
+        <v>0.007378935629743977</v>
+      </c>
+      <c r="AB34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD34" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE34" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>28.53488372093023</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>0.4987816416169121</v>
+      </c>
+      <c r="AJ34" t="n">
+        <v>28</v>
+      </c>
+      <c r="AK34" t="n">
+        <v>29</v>
+      </c>
+      <c r="AL34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN34" t="n">
+        <v>43</v>
+      </c>
+      <c r="AO34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR34" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS34" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT34" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU34" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>pg_full_ep6_nas100_rtg_late1_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>47</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>6</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G35" t="n">
+        <v>100</v>
+      </c>
+      <c r="H35" t="n">
+        <v>100</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.8977244329178085</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.5754620361328124</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.3018072524298372</v>
+      </c>
+      <c r="L35" t="n">
+        <v>11</v>
+      </c>
+      <c r="M35" t="n">
+        <v>48.16666666666666</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" t="n">
+        <v>24.96300726011395</v>
+      </c>
+      <c r="S35" t="n">
+        <v>1.590225962776458</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U35" t="n">
+        <v>1132.821846246719</v>
+      </c>
+      <c r="V35" t="n">
+        <v>0.8977244329178085</v>
+      </c>
+      <c r="W35" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0.3696195548029688</v>
+      </c>
+      <c r="AA35" t="n">
+        <v>0.01172464764772021</v>
+      </c>
+      <c r="AB35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD35" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE35" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ35" t="n">
+        <v>50</v>
+      </c>
+      <c r="AK35" t="n">
+        <v>50</v>
+      </c>
+      <c r="AL35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR35" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS35" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT35" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV35" t="inlineStr">
+        <is>
+          <t>reward_to_go</t>
+        </is>
+      </c>
+      <c r="AW35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>pg_full_ep4_nas100_late2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>47</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G36" t="n">
+        <v>100</v>
+      </c>
+      <c r="H36" t="n">
+        <v>100</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.9277247850888115</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.615855712890625</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.265774304295929</v>
+      </c>
+      <c r="L36" t="n">
+        <v>13</v>
+      </c>
+      <c r="M36" t="n">
+        <v>41.28571428571428</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R36" t="n">
+        <v>28.2383325882256</v>
+      </c>
+      <c r="S36" t="n">
+        <v>1.808217201352818</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U36" t="n">
+        <v>710.2629251480103</v>
+      </c>
+      <c r="V36" t="n">
+        <v>0.9277247850888115</v>
+      </c>
+      <c r="W36" t="n">
+        <v>0</v>
+      </c>
+      <c r="X36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0.4292762424526124</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>0.01622561783644191</v>
+      </c>
+      <c r="AB36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE36" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>42.76923076923077</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>0.4213250442347432</v>
+      </c>
+      <c r="AJ36" t="n">
+        <v>42</v>
+      </c>
+      <c r="AK36" t="n">
+        <v>43</v>
+      </c>
+      <c r="AL36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR36" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS36" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT36" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU36" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV36" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>pg_full_ep4_nas100_h64_late2_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>47</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="G37" t="n">
+        <v>100</v>
+      </c>
+      <c r="H37" t="n">
+        <v>100</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.9656392369414878</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.6264197998046874</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.2532756577156321</v>
+      </c>
+      <c r="L37" t="n">
+        <v>75</v>
+      </c>
+      <c r="M37" t="n">
+        <v>7.605263157894737</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" t="n">
+        <v>72.76864193566144</v>
+      </c>
+      <c r="S37" t="n">
+        <v>4.709534041699953</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U37" t="n">
+        <v>725.9607074260712</v>
+      </c>
+      <c r="V37" t="n">
+        <v>0.9656392369414878</v>
+      </c>
+      <c r="W37" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0.245341016575823</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>0.01806023213096329</v>
+      </c>
+      <c r="AB37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE37" t="n">
+        <v>64</v>
+      </c>
+      <c r="AF37" t="n">
+        <v>128</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH37" t="n">
+        <v>7.533333333333333</v>
+      </c>
+      <c r="AI37" t="n">
+        <v>4.151572660517404</v>
+      </c>
+      <c r="AJ37" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK37" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP37" t="n">
+        <v>38</v>
+      </c>
+      <c r="AQ37" t="n">
+        <v>0.5066666666666667</v>
+      </c>
+      <c r="AR37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS37" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT37" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV37" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW37" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add counterfactual PG controller auxiliary signal
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2980,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW37"/>
+  <dimension ref="A1:BG39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3227,6 +3227,56 @@
       <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>reward_gamma</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>aux_advantage_loss_scale</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>aux_advantage_margin</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>aux_advantage_weight_clip</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_mean</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_abs_mean</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_positive_rate</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>chosen_cf_advantage_mean</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>decision_cf_alignment_rate</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>switch_positive_advantage_rate</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>hold_negative_advantage_rate</t>
         </is>
       </c>
     </row>
@@ -3330,6 +3380,16 @@
       <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3431,6 +3491,16 @@
       <c r="AU3" t="inlineStr"/>
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
+      <c r="BE3" t="inlineStr"/>
+      <c r="BF3" t="inlineStr"/>
+      <c r="BG3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3532,6 +3602,16 @@
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="inlineStr"/>
+      <c r="BA4" t="inlineStr"/>
+      <c r="BB4" t="inlineStr"/>
+      <c r="BC4" t="inlineStr"/>
+      <c r="BD4" t="inlineStr"/>
+      <c r="BE4" t="inlineStr"/>
+      <c r="BF4" t="inlineStr"/>
+      <c r="BG4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3633,6 +3713,16 @@
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
+      <c r="BE5" t="inlineStr"/>
+      <c r="BF5" t="inlineStr"/>
+      <c r="BG5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3738,6 +3828,16 @@
       <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3843,6 +3943,16 @@
       <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3950,6 +4060,16 @@
       <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr"/>
       <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4057,6 +4177,16 @@
       <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr"/>
       <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4166,6 +4296,16 @@
       <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr"/>
       <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4283,6 +4423,16 @@
       <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4400,6 +4550,16 @@
       <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr"/>
       <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4519,6 +4679,16 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4638,6 +4808,16 @@
       <c r="AU14" t="inlineStr"/>
       <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4761,6 +4941,16 @@
       <c r="AU15" t="inlineStr"/>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4884,6 +5074,16 @@
       <c r="AU16" t="inlineStr"/>
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5007,6 +5207,16 @@
       <c r="AU17" t="inlineStr"/>
       <c r="AV17" t="inlineStr"/>
       <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5130,6 +5340,16 @@
       <c r="AU18" t="inlineStr"/>
       <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5253,6 +5473,16 @@
       <c r="AU19" t="inlineStr"/>
       <c r="AV19" t="inlineStr"/>
       <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5376,6 +5606,16 @@
       <c r="AU20" t="inlineStr"/>
       <c r="AV20" t="inlineStr"/>
       <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5499,6 +5739,16 @@
       <c r="AU21" t="inlineStr"/>
       <c r="AV21" t="inlineStr"/>
       <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+      <c r="AZ21" t="inlineStr"/>
+      <c r="BA21" t="inlineStr"/>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5644,6 +5894,16 @@
       <c r="AU22" t="inlineStr"/>
       <c r="AV22" t="inlineStr"/>
       <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5789,6 +6049,16 @@
       <c r="AU23" t="inlineStr"/>
       <c r="AV23" t="inlineStr"/>
       <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5934,6 +6204,16 @@
       <c r="AU24" t="inlineStr"/>
       <c r="AV24" t="inlineStr"/>
       <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
+      <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6085,6 +6365,16 @@
       <c r="AU25" t="inlineStr"/>
       <c r="AV25" t="inlineStr"/>
       <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+      <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6236,6 +6526,16 @@
       <c r="AU26" t="inlineStr"/>
       <c r="AV26" t="inlineStr"/>
       <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
+      <c r="BG26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6387,6 +6687,16 @@
       <c r="AU27" t="inlineStr"/>
       <c r="AV27" t="inlineStr"/>
       <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+      <c r="BA27" t="inlineStr"/>
+      <c r="BB27" t="inlineStr"/>
+      <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="inlineStr"/>
+      <c r="BF27" t="inlineStr"/>
+      <c r="BG27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6538,6 +6848,16 @@
       <c r="AU28" t="inlineStr"/>
       <c r="AV28" t="inlineStr"/>
       <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
+      <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="inlineStr"/>
+      <c r="BF28" t="inlineStr"/>
+      <c r="BG28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6689,6 +7009,16 @@
       <c r="AU29" t="inlineStr"/>
       <c r="AV29" t="inlineStr"/>
       <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="inlineStr"/>
+      <c r="BF29" t="inlineStr"/>
+      <c r="BG29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6840,6 +7170,16 @@
       <c r="AU30" t="inlineStr"/>
       <c r="AV30" t="inlineStr"/>
       <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+      <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="inlineStr"/>
+      <c r="BF30" t="inlineStr"/>
+      <c r="BG30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6991,6 +7331,16 @@
       <c r="AU31" t="inlineStr"/>
       <c r="AV31" t="inlineStr"/>
       <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
+      <c r="AZ31" t="inlineStr"/>
+      <c r="BA31" t="inlineStr"/>
+      <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="inlineStr"/>
+      <c r="BF31" t="inlineStr"/>
+      <c r="BG31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7142,6 +7492,16 @@
       <c r="AU32" t="inlineStr"/>
       <c r="AV32" t="inlineStr"/>
       <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
+      <c r="AZ32" t="inlineStr"/>
+      <c r="BA32" t="inlineStr"/>
+      <c r="BB32" t="inlineStr"/>
+      <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="inlineStr"/>
+      <c r="BF32" t="inlineStr"/>
+      <c r="BG32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7295,6 +7655,16 @@
       </c>
       <c r="AV33" t="inlineStr"/>
       <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+      <c r="BB33" t="inlineStr"/>
+      <c r="BC33" t="inlineStr"/>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="inlineStr"/>
+      <c r="BF33" t="inlineStr"/>
+      <c r="BG33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7438,6 +7808,16 @@
       </c>
       <c r="AV34" t="inlineStr"/>
       <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
+      <c r="AZ34" t="inlineStr"/>
+      <c r="BA34" t="inlineStr"/>
+      <c r="BB34" t="inlineStr"/>
+      <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr"/>
+      <c r="BE34" t="inlineStr"/>
+      <c r="BF34" t="inlineStr"/>
+      <c r="BG34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7597,6 +7977,16 @@
       <c r="AW35" t="n">
         <v>1</v>
       </c>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
+      <c r="AZ35" t="inlineStr"/>
+      <c r="BA35" t="inlineStr"/>
+      <c r="BB35" t="inlineStr"/>
+      <c r="BC35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr"/>
+      <c r="BE35" t="inlineStr"/>
+      <c r="BF35" t="inlineStr"/>
+      <c r="BG35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7756,6 +8146,16 @@
       <c r="AW36" t="n">
         <v>1</v>
       </c>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+      <c r="BB36" t="inlineStr"/>
+      <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+      <c r="BE36" t="inlineStr"/>
+      <c r="BF36" t="inlineStr"/>
+      <c r="BG36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7914,6 +8314,394 @@
       </c>
       <c r="AW37" t="n">
         <v>1</v>
+      </c>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
+      <c r="AZ37" t="inlineStr"/>
+      <c r="BA37" t="inlineStr"/>
+      <c r="BB37" t="inlineStr"/>
+      <c r="BC37" t="inlineStr"/>
+      <c r="BD37" t="inlineStr"/>
+      <c r="BE37" t="inlineStr"/>
+      <c r="BF37" t="inlineStr"/>
+      <c r="BG37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>pg_smoke_auxcf_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>47</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G38" t="n">
+        <v>100</v>
+      </c>
+      <c r="H38" t="n">
+        <v>100</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2.978769103847668</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.2673975830078126</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.07820563302977675</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" t="n">
+        <v>4.685821387916803</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0.2759422055387404</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U38" t="n">
+        <v>130.7273421287537</v>
+      </c>
+      <c r="V38" t="n">
+        <v>2.978769103847668</v>
+      </c>
+      <c r="W38" t="n">
+        <v>0</v>
+      </c>
+      <c r="X38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0.4242733739713421</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>0.01615732979889099</v>
+      </c>
+      <c r="AB38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD38" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE38" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF38" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH38" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="AI38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ38" t="n">
+        <v>43</v>
+      </c>
+      <c r="AK38" t="n">
+        <v>44</v>
+      </c>
+      <c r="AL38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR38" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT38" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ38" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA38" t="n">
+        <v>-7.076903441839767e-05</v>
+      </c>
+      <c r="BB38" t="n">
+        <v>0.003309554941447683</v>
+      </c>
+      <c r="BC38" t="n">
+        <v>0.4672131147540984</v>
+      </c>
+      <c r="BD38" t="n">
+        <v>7.030856029247888e-05</v>
+      </c>
+      <c r="BE38" t="n">
+        <v>0.5327868852459017</v>
+      </c>
+      <c r="BF38" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BG38" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>pg_smoke_auxcf_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>77</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G39" t="n">
+        <v>100</v>
+      </c>
+      <c r="H39" t="n">
+        <v>100</v>
+      </c>
+      <c r="I39" t="n">
+        <v>2.299238280181702</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.3393822021484374</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.1166293682142446</v>
+      </c>
+      <c r="L39" t="n">
+        <v>4</v>
+      </c>
+      <c r="M39" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="n">
+        <v>8.01088716648519</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0.4895865195721854</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U39" t="n">
+        <v>134.3627624511719</v>
+      </c>
+      <c r="V39" t="n">
+        <v>1.799238280181702</v>
+      </c>
+      <c r="W39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0.3512284095912915</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>0.01247940629365898</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE39" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF39" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH39" t="n">
+        <v>27</v>
+      </c>
+      <c r="AI39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ39" t="n">
+        <v>27</v>
+      </c>
+      <c r="AK39" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN39" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV39" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX39" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AY39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA39" t="n">
+        <v>0.0006717431714260501</v>
+      </c>
+      <c r="BB39" t="n">
+        <v>0.007777126970628662</v>
+      </c>
+      <c r="BC39" t="n">
+        <v>0.4741379310344828</v>
+      </c>
+      <c r="BD39" t="n">
+        <v>-0.0005026316513098648</v>
+      </c>
+      <c r="BE39" t="n">
+        <v>0.5086206896551724</v>
+      </c>
+      <c r="BF39" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BG39" t="n">
+        <v>0.5178571428571429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Train PG controller on penalized objective
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2980,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG39"/>
+  <dimension ref="A1:BI42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3277,6 +3277,16 @@
       <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>hold_negative_advantage_rate</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>mask_hold_age_feature</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>supervised_pretrain_episodes</t>
         </is>
       </c>
     </row>
@@ -3390,6 +3400,8 @@
       <c r="BE2" t="inlineStr"/>
       <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3501,6 +3513,8 @@
       <c r="BE3" t="inlineStr"/>
       <c r="BF3" t="inlineStr"/>
       <c r="BG3" t="inlineStr"/>
+      <c r="BH3" t="inlineStr"/>
+      <c r="BI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3612,6 +3626,8 @@
       <c r="BE4" t="inlineStr"/>
       <c r="BF4" t="inlineStr"/>
       <c r="BG4" t="inlineStr"/>
+      <c r="BH4" t="inlineStr"/>
+      <c r="BI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3723,6 +3739,8 @@
       <c r="BE5" t="inlineStr"/>
       <c r="BF5" t="inlineStr"/>
       <c r="BG5" t="inlineStr"/>
+      <c r="BH5" t="inlineStr"/>
+      <c r="BI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3838,6 +3856,8 @@
       <c r="BE6" t="inlineStr"/>
       <c r="BF6" t="inlineStr"/>
       <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+      <c r="BI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3953,6 +3973,8 @@
       <c r="BE7" t="inlineStr"/>
       <c r="BF7" t="inlineStr"/>
       <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+      <c r="BI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4070,6 +4092,8 @@
       <c r="BE8" t="inlineStr"/>
       <c r="BF8" t="inlineStr"/>
       <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4187,6 +4211,8 @@
       <c r="BE9" t="inlineStr"/>
       <c r="BF9" t="inlineStr"/>
       <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
+      <c r="BI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4306,6 +4332,8 @@
       <c r="BE10" t="inlineStr"/>
       <c r="BF10" t="inlineStr"/>
       <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
+      <c r="BI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4433,6 +4461,8 @@
       <c r="BE11" t="inlineStr"/>
       <c r="BF11" t="inlineStr"/>
       <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr"/>
+      <c r="BI11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4560,6 +4590,8 @@
       <c r="BE12" t="inlineStr"/>
       <c r="BF12" t="inlineStr"/>
       <c r="BG12" t="inlineStr"/>
+      <c r="BH12" t="inlineStr"/>
+      <c r="BI12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4689,6 +4721,8 @@
       <c r="BE13" t="inlineStr"/>
       <c r="BF13" t="inlineStr"/>
       <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4818,6 +4852,8 @@
       <c r="BE14" t="inlineStr"/>
       <c r="BF14" t="inlineStr"/>
       <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
+      <c r="BI14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4951,6 +4987,8 @@
       <c r="BE15" t="inlineStr"/>
       <c r="BF15" t="inlineStr"/>
       <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
+      <c r="BI15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5084,6 +5122,8 @@
       <c r="BE16" t="inlineStr"/>
       <c r="BF16" t="inlineStr"/>
       <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr"/>
+      <c r="BI16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5217,6 +5257,8 @@
       <c r="BE17" t="inlineStr"/>
       <c r="BF17" t="inlineStr"/>
       <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5350,6 +5392,8 @@
       <c r="BE18" t="inlineStr"/>
       <c r="BF18" t="inlineStr"/>
       <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5483,6 +5527,8 @@
       <c r="BE19" t="inlineStr"/>
       <c r="BF19" t="inlineStr"/>
       <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5616,6 +5662,8 @@
       <c r="BE20" t="inlineStr"/>
       <c r="BF20" t="inlineStr"/>
       <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5749,6 +5797,8 @@
       <c r="BE21" t="inlineStr"/>
       <c r="BF21" t="inlineStr"/>
       <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5904,6 +5954,8 @@
       <c r="BE22" t="inlineStr"/>
       <c r="BF22" t="inlineStr"/>
       <c r="BG22" t="inlineStr"/>
+      <c r="BH22" t="inlineStr"/>
+      <c r="BI22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6059,6 +6111,8 @@
       <c r="BE23" t="inlineStr"/>
       <c r="BF23" t="inlineStr"/>
       <c r="BG23" t="inlineStr"/>
+      <c r="BH23" t="inlineStr"/>
+      <c r="BI23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6214,6 +6268,8 @@
       <c r="BE24" t="inlineStr"/>
       <c r="BF24" t="inlineStr"/>
       <c r="BG24" t="inlineStr"/>
+      <c r="BH24" t="inlineStr"/>
+      <c r="BI24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6375,6 +6431,8 @@
       <c r="BE25" t="inlineStr"/>
       <c r="BF25" t="inlineStr"/>
       <c r="BG25" t="inlineStr"/>
+      <c r="BH25" t="inlineStr"/>
+      <c r="BI25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6536,6 +6594,8 @@
       <c r="BE26" t="inlineStr"/>
       <c r="BF26" t="inlineStr"/>
       <c r="BG26" t="inlineStr"/>
+      <c r="BH26" t="inlineStr"/>
+      <c r="BI26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6697,6 +6757,8 @@
       <c r="BE27" t="inlineStr"/>
       <c r="BF27" t="inlineStr"/>
       <c r="BG27" t="inlineStr"/>
+      <c r="BH27" t="inlineStr"/>
+      <c r="BI27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6858,6 +6920,8 @@
       <c r="BE28" t="inlineStr"/>
       <c r="BF28" t="inlineStr"/>
       <c r="BG28" t="inlineStr"/>
+      <c r="BH28" t="inlineStr"/>
+      <c r="BI28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7019,6 +7083,8 @@
       <c r="BE29" t="inlineStr"/>
       <c r="BF29" t="inlineStr"/>
       <c r="BG29" t="inlineStr"/>
+      <c r="BH29" t="inlineStr"/>
+      <c r="BI29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7180,6 +7246,8 @@
       <c r="BE30" t="inlineStr"/>
       <c r="BF30" t="inlineStr"/>
       <c r="BG30" t="inlineStr"/>
+      <c r="BH30" t="inlineStr"/>
+      <c r="BI30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7341,6 +7409,8 @@
       <c r="BE31" t="inlineStr"/>
       <c r="BF31" t="inlineStr"/>
       <c r="BG31" t="inlineStr"/>
+      <c r="BH31" t="inlineStr"/>
+      <c r="BI31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7502,6 +7572,8 @@
       <c r="BE32" t="inlineStr"/>
       <c r="BF32" t="inlineStr"/>
       <c r="BG32" t="inlineStr"/>
+      <c r="BH32" t="inlineStr"/>
+      <c r="BI32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7665,6 +7737,8 @@
       <c r="BE33" t="inlineStr"/>
       <c r="BF33" t="inlineStr"/>
       <c r="BG33" t="inlineStr"/>
+      <c r="BH33" t="inlineStr"/>
+      <c r="BI33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7818,6 +7892,8 @@
       <c r="BE34" t="inlineStr"/>
       <c r="BF34" t="inlineStr"/>
       <c r="BG34" t="inlineStr"/>
+      <c r="BH34" t="inlineStr"/>
+      <c r="BI34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7987,6 +8063,8 @@
       <c r="BE35" t="inlineStr"/>
       <c r="BF35" t="inlineStr"/>
       <c r="BG35" t="inlineStr"/>
+      <c r="BH35" t="inlineStr"/>
+      <c r="BI35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8156,6 +8234,8 @@
       <c r="BE36" t="inlineStr"/>
       <c r="BF36" t="inlineStr"/>
       <c r="BG36" t="inlineStr"/>
+      <c r="BH36" t="inlineStr"/>
+      <c r="BI36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8325,6 +8405,8 @@
       <c r="BE37" t="inlineStr"/>
       <c r="BF37" t="inlineStr"/>
       <c r="BG37" t="inlineStr"/>
+      <c r="BH37" t="inlineStr"/>
+      <c r="BI37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8514,6 +8596,8 @@
       <c r="BG38" t="n">
         <v>0.5333333333333333</v>
       </c>
+      <c r="BH38" t="inlineStr"/>
+      <c r="BI38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8702,6 +8786,591 @@
       </c>
       <c r="BG39" t="n">
         <v>0.5178571428571429</v>
+      </c>
+      <c r="BH39" t="inlineStr"/>
+      <c r="BI39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>pg_smoke_maskage_aux5_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>77</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G40" t="n">
+        <v>100</v>
+      </c>
+      <c r="H40" t="n">
+        <v>100</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L40" t="n">
+        <v>3</v>
+      </c>
+      <c r="M40" t="n">
+        <v>29</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U40" t="n">
+        <v>100.2985002994537</v>
+      </c>
+      <c r="V40" t="n">
+        <v>-1.282923151096803</v>
+      </c>
+      <c r="W40" t="n">
+        <v>4</v>
+      </c>
+      <c r="X40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0.3646379749788421</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>0.01267093206372331</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>0.9738566478093466</v>
+      </c>
+      <c r="AC40" t="n">
+        <v>0.02614333232243856</v>
+      </c>
+      <c r="AD40" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE40" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF40" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH40" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ40" t="n">
+        <v>30</v>
+      </c>
+      <c r="AK40" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN40" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU40" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV40" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW40" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX40" t="n">
+        <v>5</v>
+      </c>
+      <c r="AY40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA40" t="n">
+        <v>-0.0001386595410214544</v>
+      </c>
+      <c r="BB40" t="n">
+        <v>0.007125838668735954</v>
+      </c>
+      <c r="BC40" t="n">
+        <v>0.456896551724138</v>
+      </c>
+      <c r="BD40" t="n">
+        <v>0.0001804590725002746</v>
+      </c>
+      <c r="BE40" t="n">
+        <v>0.5344827586206896</v>
+      </c>
+      <c r="BF40" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="BG40" t="n">
+        <v>0.5398230088495575</v>
+      </c>
+      <c r="BH40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>pg_smoke_pretrain5_aux1_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>77</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G41" t="n">
+        <v>100</v>
+      </c>
+      <c r="H41" t="n">
+        <v>100</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.717076848903197</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.4394011230468751</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.1925831512503035</v>
+      </c>
+      <c r="L41" t="n">
+        <v>3</v>
+      </c>
+      <c r="M41" t="n">
+        <v>29</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="n">
+        <v>7.917359989136457</v>
+      </c>
+      <c r="S41" t="n">
+        <v>0.5189761720830575</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U41" t="n">
+        <v>142.5196237564087</v>
+      </c>
+      <c r="V41" t="n">
+        <v>-1.282923151096803</v>
+      </c>
+      <c r="W41" t="n">
+        <v>4</v>
+      </c>
+      <c r="X41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0.4306583626452705</v>
+      </c>
+      <c r="AA41" t="n">
+        <v>0.01733381147770321</v>
+      </c>
+      <c r="AB41" t="n">
+        <v>0.9808106422424316</v>
+      </c>
+      <c r="AC41" t="n">
+        <v>0.01918940308193366</v>
+      </c>
+      <c r="AD41" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE41" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF41" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG41" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH41" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ41" t="n">
+        <v>30</v>
+      </c>
+      <c r="AK41" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL41" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN41" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR41" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU41" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV41" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX41" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA41" t="n">
+        <v>-0.0001386595410214544</v>
+      </c>
+      <c r="BB41" t="n">
+        <v>0.007125838668735954</v>
+      </c>
+      <c r="BC41" t="n">
+        <v>0.456896551724138</v>
+      </c>
+      <c r="BD41" t="n">
+        <v>0.0001804590725002746</v>
+      </c>
+      <c r="BE41" t="n">
+        <v>0.5344827586206896</v>
+      </c>
+      <c r="BF41" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="BG41" t="n">
+        <v>0.5398230088495575</v>
+      </c>
+      <c r="BH41" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI41" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>pg_smoke_objective_train_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>77</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G42" t="n">
+        <v>100</v>
+      </c>
+      <c r="H42" t="n">
+        <v>100</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2.164669923688698</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.3160112304687499</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.1717557738494409</v>
+      </c>
+      <c r="L42" t="n">
+        <v>4</v>
+      </c>
+      <c r="M42" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" t="n">
+        <v>7.988446166738868</v>
+      </c>
+      <c r="S42" t="n">
+        <v>0.48322448975523</v>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U42" t="n">
+        <v>128.5693693161011</v>
+      </c>
+      <c r="V42" t="n">
+        <v>1.664669923688698</v>
+      </c>
+      <c r="W42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X42" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>0.3545865642452805</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>0.01251018038463025</v>
+      </c>
+      <c r="AB42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD42" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE42" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF42" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH42" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="AI42" t="n">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="AJ42" t="n">
+        <v>26</v>
+      </c>
+      <c r="AK42" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO42" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR42" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS42" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU42" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV42" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA42" t="n">
+        <v>0.0006148732861439729</v>
+      </c>
+      <c r="BB42" t="n">
+        <v>0.006859226373088514</v>
+      </c>
+      <c r="BC42" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD42" t="n">
+        <v>-0.00049106626578703</v>
+      </c>
+      <c r="BE42" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BF42" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BG42" t="n">
+        <v>0.5267857142857143</v>
+      </c>
+      <c r="BH42" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI42" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add boundary diagnostics to PG controller training
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2980,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BI42"/>
+  <dimension ref="A1:BK50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3287,6 +3287,16 @@
       <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>supervised_pretrain_episodes</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>hard_boundary_mask</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>min_boundary_penalty</t>
         </is>
       </c>
     </row>
@@ -3402,6 +3412,8 @@
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3515,6 +3527,8 @@
       <c r="BG3" t="inlineStr"/>
       <c r="BH3" t="inlineStr"/>
       <c r="BI3" t="inlineStr"/>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3628,6 +3642,8 @@
       <c r="BG4" t="inlineStr"/>
       <c r="BH4" t="inlineStr"/>
       <c r="BI4" t="inlineStr"/>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3741,6 +3757,8 @@
       <c r="BG5" t="inlineStr"/>
       <c r="BH5" t="inlineStr"/>
       <c r="BI5" t="inlineStr"/>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3858,6 +3876,8 @@
       <c r="BG6" t="inlineStr"/>
       <c r="BH6" t="inlineStr"/>
       <c r="BI6" t="inlineStr"/>
+      <c r="BJ6" t="inlineStr"/>
+      <c r="BK6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3975,6 +3995,8 @@
       <c r="BG7" t="inlineStr"/>
       <c r="BH7" t="inlineStr"/>
       <c r="BI7" t="inlineStr"/>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4094,6 +4116,8 @@
       <c r="BG8" t="inlineStr"/>
       <c r="BH8" t="inlineStr"/>
       <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4213,6 +4237,8 @@
       <c r="BG9" t="inlineStr"/>
       <c r="BH9" t="inlineStr"/>
       <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4334,6 +4360,8 @@
       <c r="BG10" t="inlineStr"/>
       <c r="BH10" t="inlineStr"/>
       <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4463,6 +4491,8 @@
       <c r="BG11" t="inlineStr"/>
       <c r="BH11" t="inlineStr"/>
       <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4592,6 +4622,8 @@
       <c r="BG12" t="inlineStr"/>
       <c r="BH12" t="inlineStr"/>
       <c r="BI12" t="inlineStr"/>
+      <c r="BJ12" t="inlineStr"/>
+      <c r="BK12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4723,6 +4755,8 @@
       <c r="BG13" t="inlineStr"/>
       <c r="BH13" t="inlineStr"/>
       <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4854,6 +4888,8 @@
       <c r="BG14" t="inlineStr"/>
       <c r="BH14" t="inlineStr"/>
       <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4989,6 +5025,8 @@
       <c r="BG15" t="inlineStr"/>
       <c r="BH15" t="inlineStr"/>
       <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5124,6 +5162,8 @@
       <c r="BG16" t="inlineStr"/>
       <c r="BH16" t="inlineStr"/>
       <c r="BI16" t="inlineStr"/>
+      <c r="BJ16" t="inlineStr"/>
+      <c r="BK16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5259,6 +5299,8 @@
       <c r="BG17" t="inlineStr"/>
       <c r="BH17" t="inlineStr"/>
       <c r="BI17" t="inlineStr"/>
+      <c r="BJ17" t="inlineStr"/>
+      <c r="BK17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5394,6 +5436,8 @@
       <c r="BG18" t="inlineStr"/>
       <c r="BH18" t="inlineStr"/>
       <c r="BI18" t="inlineStr"/>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5529,6 +5573,8 @@
       <c r="BG19" t="inlineStr"/>
       <c r="BH19" t="inlineStr"/>
       <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5664,6 +5710,8 @@
       <c r="BG20" t="inlineStr"/>
       <c r="BH20" t="inlineStr"/>
       <c r="BI20" t="inlineStr"/>
+      <c r="BJ20" t="inlineStr"/>
+      <c r="BK20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5799,6 +5847,8 @@
       <c r="BG21" t="inlineStr"/>
       <c r="BH21" t="inlineStr"/>
       <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="inlineStr"/>
+      <c r="BK21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5956,6 +6006,8 @@
       <c r="BG22" t="inlineStr"/>
       <c r="BH22" t="inlineStr"/>
       <c r="BI22" t="inlineStr"/>
+      <c r="BJ22" t="inlineStr"/>
+      <c r="BK22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6113,6 +6165,8 @@
       <c r="BG23" t="inlineStr"/>
       <c r="BH23" t="inlineStr"/>
       <c r="BI23" t="inlineStr"/>
+      <c r="BJ23" t="inlineStr"/>
+      <c r="BK23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6270,6 +6324,8 @@
       <c r="BG24" t="inlineStr"/>
       <c r="BH24" t="inlineStr"/>
       <c r="BI24" t="inlineStr"/>
+      <c r="BJ24" t="inlineStr"/>
+      <c r="BK24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6433,6 +6489,8 @@
       <c r="BG25" t="inlineStr"/>
       <c r="BH25" t="inlineStr"/>
       <c r="BI25" t="inlineStr"/>
+      <c r="BJ25" t="inlineStr"/>
+      <c r="BK25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6596,6 +6654,8 @@
       <c r="BG26" t="inlineStr"/>
       <c r="BH26" t="inlineStr"/>
       <c r="BI26" t="inlineStr"/>
+      <c r="BJ26" t="inlineStr"/>
+      <c r="BK26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6759,6 +6819,8 @@
       <c r="BG27" t="inlineStr"/>
       <c r="BH27" t="inlineStr"/>
       <c r="BI27" t="inlineStr"/>
+      <c r="BJ27" t="inlineStr"/>
+      <c r="BK27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6922,6 +6984,8 @@
       <c r="BG28" t="inlineStr"/>
       <c r="BH28" t="inlineStr"/>
       <c r="BI28" t="inlineStr"/>
+      <c r="BJ28" t="inlineStr"/>
+      <c r="BK28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7085,6 +7149,8 @@
       <c r="BG29" t="inlineStr"/>
       <c r="BH29" t="inlineStr"/>
       <c r="BI29" t="inlineStr"/>
+      <c r="BJ29" t="inlineStr"/>
+      <c r="BK29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7248,6 +7314,8 @@
       <c r="BG30" t="inlineStr"/>
       <c r="BH30" t="inlineStr"/>
       <c r="BI30" t="inlineStr"/>
+      <c r="BJ30" t="inlineStr"/>
+      <c r="BK30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7411,6 +7479,8 @@
       <c r="BG31" t="inlineStr"/>
       <c r="BH31" t="inlineStr"/>
       <c r="BI31" t="inlineStr"/>
+      <c r="BJ31" t="inlineStr"/>
+      <c r="BK31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7574,6 +7644,8 @@
       <c r="BG32" t="inlineStr"/>
       <c r="BH32" t="inlineStr"/>
       <c r="BI32" t="inlineStr"/>
+      <c r="BJ32" t="inlineStr"/>
+      <c r="BK32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7739,6 +7811,8 @@
       <c r="BG33" t="inlineStr"/>
       <c r="BH33" t="inlineStr"/>
       <c r="BI33" t="inlineStr"/>
+      <c r="BJ33" t="inlineStr"/>
+      <c r="BK33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7894,6 +7968,8 @@
       <c r="BG34" t="inlineStr"/>
       <c r="BH34" t="inlineStr"/>
       <c r="BI34" t="inlineStr"/>
+      <c r="BJ34" t="inlineStr"/>
+      <c r="BK34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8065,6 +8141,8 @@
       <c r="BG35" t="inlineStr"/>
       <c r="BH35" t="inlineStr"/>
       <c r="BI35" t="inlineStr"/>
+      <c r="BJ35" t="inlineStr"/>
+      <c r="BK35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8236,6 +8314,8 @@
       <c r="BG36" t="inlineStr"/>
       <c r="BH36" t="inlineStr"/>
       <c r="BI36" t="inlineStr"/>
+      <c r="BJ36" t="inlineStr"/>
+      <c r="BK36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8407,6 +8487,8 @@
       <c r="BG37" t="inlineStr"/>
       <c r="BH37" t="inlineStr"/>
       <c r="BI37" t="inlineStr"/>
+      <c r="BJ37" t="inlineStr"/>
+      <c r="BK37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8598,6 +8680,8 @@
       </c>
       <c r="BH38" t="inlineStr"/>
       <c r="BI38" t="inlineStr"/>
+      <c r="BJ38" t="inlineStr"/>
+      <c r="BK38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8789,6 +8873,8 @@
       </c>
       <c r="BH39" t="inlineStr"/>
       <c r="BI39" t="inlineStr"/>
+      <c r="BJ39" t="inlineStr"/>
+      <c r="BK39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8982,6 +9068,8 @@
         <v>1</v>
       </c>
       <c r="BI40" t="inlineStr"/>
+      <c r="BJ40" t="inlineStr"/>
+      <c r="BK40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9177,6 +9265,8 @@
       <c r="BI41" t="n">
         <v>5</v>
       </c>
+      <c r="BJ41" t="inlineStr"/>
+      <c r="BK41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9371,6 +9461,1604 @@
       </c>
       <c r="BI42" t="n">
         <v>0</v>
+      </c>
+      <c r="BJ42" t="inlineStr"/>
+      <c r="BK42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>pg_full_objective_train_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>77</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>8</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G43" t="n">
+        <v>100</v>
+      </c>
+      <c r="H43" t="n">
+        <v>100</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.5459325402401566</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.2195341796875001</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.3014408640723663</v>
+      </c>
+      <c r="L43" t="n">
+        <v>21</v>
+      </c>
+      <c r="M43" t="n">
+        <v>22.04545454545455</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" t="n">
+        <v>41.82066904194653</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.967710629018256</v>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U43" t="n">
+        <v>1881.837561607361</v>
+      </c>
+      <c r="V43" t="n">
+        <v>0.5459325402401566</v>
+      </c>
+      <c r="W43" t="n">
+        <v>0</v>
+      </c>
+      <c r="X43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>0.373471082545356</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>0.01415989304149754</v>
+      </c>
+      <c r="AB43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD43" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE43" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF43" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH43" t="n">
+        <v>22.80952380952381</v>
+      </c>
+      <c r="AI43" t="n">
+        <v>1.401327520910682</v>
+      </c>
+      <c r="AJ43" t="n">
+        <v>20</v>
+      </c>
+      <c r="AK43" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR43" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU43" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV43" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX43" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA43" t="n">
+        <v>-0.0002359449094732666</v>
+      </c>
+      <c r="BB43" t="n">
+        <v>0.006182390386202689</v>
+      </c>
+      <c r="BC43" t="n">
+        <v>0.4824742268041237</v>
+      </c>
+      <c r="BD43" t="n">
+        <v>0.00029951964316592</v>
+      </c>
+      <c r="BE43" t="n">
+        <v>0.5154639175257731</v>
+      </c>
+      <c r="BF43" t="n">
+        <v>0.4761904761904762</v>
+      </c>
+      <c r="BG43" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BH43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI43" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ43" t="inlineStr"/>
+      <c r="BK43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>pg_full_objective_train_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>47</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>8</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G44" t="n">
+        <v>100</v>
+      </c>
+      <c r="H44" t="n">
+        <v>100</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.07551331377294</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.7685574951171874</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.2896415739896901</v>
+      </c>
+      <c r="L44" t="n">
+        <v>14</v>
+      </c>
+      <c r="M44" t="n">
+        <v>38.53333333333333</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" t="n">
+        <v>26.86953561194241</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.78496674154303</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U44" t="n">
+        <v>1922.280446052551</v>
+      </c>
+      <c r="V44" t="n">
+        <v>1.07551331377294</v>
+      </c>
+      <c r="W44" t="n">
+        <v>0</v>
+      </c>
+      <c r="X44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>0.4282495180454273</v>
+      </c>
+      <c r="AA44" t="n">
+        <v>0.01623926644564652</v>
+      </c>
+      <c r="AB44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD44" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE44" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF44" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG44" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH44" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="AI44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AJ44" t="n">
+        <v>38</v>
+      </c>
+      <c r="AK44" t="n">
+        <v>39</v>
+      </c>
+      <c r="AL44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR44" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT44" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU44" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV44" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX44" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA44" t="n">
+        <v>-8.926338970960862e-05</v>
+      </c>
+      <c r="BB44" t="n">
+        <v>0.003770173678761123</v>
+      </c>
+      <c r="BC44" t="n">
+        <v>0.4757785467128028</v>
+      </c>
+      <c r="BD44" t="n">
+        <v>0.0001192098302375138</v>
+      </c>
+      <c r="BE44" t="n">
+        <v>0.5311418685121108</v>
+      </c>
+      <c r="BF44" t="n">
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="BG44" t="n">
+        <v>0.5283687943262412</v>
+      </c>
+      <c r="BH44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI44" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ44" t="inlineStr"/>
+      <c r="BK44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>pg_smoke_hardmask_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>47</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G45" t="n">
+        <v>100</v>
+      </c>
+      <c r="H45" t="n">
+        <v>100</v>
+      </c>
+      <c r="I45" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L45" t="n">
+        <v>24</v>
+      </c>
+      <c r="M45" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U45" t="n">
+        <v>114.6443266868591</v>
+      </c>
+      <c r="V45" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="W45" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>0.1079058388217551</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE45" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP45" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV45" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX45" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA45" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB45" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC45" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD45" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE45" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF45" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG45" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>pg_smoke_hardmask_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>77</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G46" t="n">
+        <v>100</v>
+      </c>
+      <c r="H46" t="n">
+        <v>100</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2.164669923688698</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.3160112304687499</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.1717557738494409</v>
+      </c>
+      <c r="L46" t="n">
+        <v>4</v>
+      </c>
+      <c r="M46" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" t="n">
+        <v>7.988446166738868</v>
+      </c>
+      <c r="S46" t="n">
+        <v>0.48322448975523</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U46" t="n">
+        <v>121.6785888671875</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.664669923688698</v>
+      </c>
+      <c r="W46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>0.3527574772978651</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG46" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH46" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>26</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO46" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS46" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV46" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA46" t="n">
+        <v>0.0006148732861439729</v>
+      </c>
+      <c r="BB46" t="n">
+        <v>0.006859226373088514</v>
+      </c>
+      <c r="BC46" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD46" t="n">
+        <v>-0.00049106626578703</v>
+      </c>
+      <c r="BE46" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BF46" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BG46" t="n">
+        <v>0.5267857142857143</v>
+      </c>
+      <c r="BH46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI46" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>pg_smoke_hardmask_minguard_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>47</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G47" t="n">
+        <v>100</v>
+      </c>
+      <c r="H47" t="n">
+        <v>100</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L47" t="n">
+        <v>24</v>
+      </c>
+      <c r="M47" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S47" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U47" t="n">
+        <v>120.5931475162506</v>
+      </c>
+      <c r="V47" t="n">
+        <v>0.8911775512134743</v>
+      </c>
+      <c r="W47" t="n">
+        <v>2</v>
+      </c>
+      <c r="X47" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>0.1079294862317257</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG47" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH47" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ47" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK47" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP47" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV47" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA47" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB47" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC47" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD47" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE47" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF47" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK47" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>pg_smoke_hardmask_minguard_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>77</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G48" t="n">
+        <v>100</v>
+      </c>
+      <c r="H48" t="n">
+        <v>100</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.164669923688698</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.3160112304687499</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.1717557738494409</v>
+      </c>
+      <c r="L48" t="n">
+        <v>4</v>
+      </c>
+      <c r="M48" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" t="n">
+        <v>7.988446166738868</v>
+      </c>
+      <c r="S48" t="n">
+        <v>0.48322448975523</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U48" t="n">
+        <v>137.0306694507599</v>
+      </c>
+      <c r="V48" t="n">
+        <v>1.664669923688698</v>
+      </c>
+      <c r="W48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X48" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>0.3527006175497482</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE48" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH48" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="AI48" t="n">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>26</v>
+      </c>
+      <c r="AK48" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS48" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV48" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX48" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA48" t="n">
+        <v>0.0006148732861439729</v>
+      </c>
+      <c r="BB48" t="n">
+        <v>0.006859226373088514</v>
+      </c>
+      <c r="BC48" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD48" t="n">
+        <v>-0.00049106626578703</v>
+      </c>
+      <c r="BE48" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BF48" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BG48" t="n">
+        <v>0.5267857142857143</v>
+      </c>
+      <c r="BH48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI48" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK48" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>pg_smoke_softbias10_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>47</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G49" t="n">
+        <v>100</v>
+      </c>
+      <c r="H49" t="n">
+        <v>100</v>
+      </c>
+      <c r="I49" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L49" t="n">
+        <v>24</v>
+      </c>
+      <c r="M49" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N49" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U49" t="n">
+        <v>120.4937825202942</v>
+      </c>
+      <c r="V49" t="n">
+        <v>0.8911775512134743</v>
+      </c>
+      <c r="W49" t="n">
+        <v>2</v>
+      </c>
+      <c r="X49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>0.1079770702214222</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>5.51822711862101e-05</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG49" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH49" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK49" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP49" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV49" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA49" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB49" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC49" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD49" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE49" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF49" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG49" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ49" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK49" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>pg_smoke_softbias10_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>77</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G50" t="n">
+        <v>100</v>
+      </c>
+      <c r="H50" t="n">
+        <v>100</v>
+      </c>
+      <c r="I50" t="n">
+        <v>2.164669923688698</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.3160112304687499</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.1717557738494409</v>
+      </c>
+      <c r="L50" t="n">
+        <v>4</v>
+      </c>
+      <c r="M50" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N50" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" t="n">
+        <v>7.988446166738868</v>
+      </c>
+      <c r="S50" t="n">
+        <v>0.48322448975523</v>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U50" t="n">
+        <v>128.2822382450104</v>
+      </c>
+      <c r="V50" t="n">
+        <v>1.664669923688698</v>
+      </c>
+      <c r="W50" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X50" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>0.3526985980696705</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>3.147061267684746e-05</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG50" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH50" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>26</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>27</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO50" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AP50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR50" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS50" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT50" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU50" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV50" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA50" t="n">
+        <v>0.0006148732861439729</v>
+      </c>
+      <c r="BB50" t="n">
+        <v>0.006859226373088514</v>
+      </c>
+      <c r="BC50" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD50" t="n">
+        <v>-0.00049106626578703</v>
+      </c>
+      <c r="BE50" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BF50" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BG50" t="n">
+        <v>0.5267857142857143</v>
+      </c>
+      <c r="BH50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ50" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK50" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add risk gated compact PG controller embeddings
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2980,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK50"/>
+  <dimension ref="A1:BU56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3297,6 +3297,56 @@
       <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>min_boundary_penalty</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>use_risk_gate</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>risk_gate_floor</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>risk_gate_prior_scale</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>embedding_mode</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>gate_mean</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>gate_std</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>gate_max</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>gate_live</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>gate_switch_minus_hold</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>gate_top5_mass</t>
         </is>
       </c>
     </row>
@@ -3414,6 +3464,16 @@
       <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3529,6 +3589,16 @@
       <c r="BI3" t="inlineStr"/>
       <c r="BJ3" t="inlineStr"/>
       <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="inlineStr"/>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr"/>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3644,6 +3714,16 @@
       <c r="BI4" t="inlineStr"/>
       <c r="BJ4" t="inlineStr"/>
       <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="inlineStr"/>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3759,6 +3839,16 @@
       <c r="BI5" t="inlineStr"/>
       <c r="BJ5" t="inlineStr"/>
       <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="inlineStr"/>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr"/>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3878,6 +3968,16 @@
       <c r="BI6" t="inlineStr"/>
       <c r="BJ6" t="inlineStr"/>
       <c r="BK6" t="inlineStr"/>
+      <c r="BL6" t="inlineStr"/>
+      <c r="BM6" t="inlineStr"/>
+      <c r="BN6" t="inlineStr"/>
+      <c r="BO6" t="inlineStr"/>
+      <c r="BP6" t="inlineStr"/>
+      <c r="BQ6" t="inlineStr"/>
+      <c r="BR6" t="inlineStr"/>
+      <c r="BS6" t="inlineStr"/>
+      <c r="BT6" t="inlineStr"/>
+      <c r="BU6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3997,6 +4097,16 @@
       <c r="BI7" t="inlineStr"/>
       <c r="BJ7" t="inlineStr"/>
       <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="inlineStr"/>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr"/>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4118,6 +4228,16 @@
       <c r="BI8" t="inlineStr"/>
       <c r="BJ8" t="inlineStr"/>
       <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4239,6 +4359,16 @@
       <c r="BI9" t="inlineStr"/>
       <c r="BJ9" t="inlineStr"/>
       <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4362,6 +4492,16 @@
       <c r="BI10" t="inlineStr"/>
       <c r="BJ10" t="inlineStr"/>
       <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4493,6 +4633,16 @@
       <c r="BI11" t="inlineStr"/>
       <c r="BJ11" t="inlineStr"/>
       <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4624,6 +4774,16 @@
       <c r="BI12" t="inlineStr"/>
       <c r="BJ12" t="inlineStr"/>
       <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr"/>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4757,6 +4917,16 @@
       <c r="BI13" t="inlineStr"/>
       <c r="BJ13" t="inlineStr"/>
       <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4890,6 +5060,16 @@
       <c r="BI14" t="inlineStr"/>
       <c r="BJ14" t="inlineStr"/>
       <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5027,6 +5207,16 @@
       <c r="BI15" t="inlineStr"/>
       <c r="BJ15" t="inlineStr"/>
       <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="inlineStr"/>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5164,6 +5354,16 @@
       <c r="BI16" t="inlineStr"/>
       <c r="BJ16" t="inlineStr"/>
       <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5301,6 +5501,16 @@
       <c r="BI17" t="inlineStr"/>
       <c r="BJ17" t="inlineStr"/>
       <c r="BK17" t="inlineStr"/>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
+      <c r="BO17" t="inlineStr"/>
+      <c r="BP17" t="inlineStr"/>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5438,6 +5648,16 @@
       <c r="BI18" t="inlineStr"/>
       <c r="BJ18" t="inlineStr"/>
       <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5575,6 +5795,16 @@
       <c r="BI19" t="inlineStr"/>
       <c r="BJ19" t="inlineStr"/>
       <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr"/>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr"/>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5712,6 +5942,16 @@
       <c r="BI20" t="inlineStr"/>
       <c r="BJ20" t="inlineStr"/>
       <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="inlineStr"/>
+      <c r="BP20" t="inlineStr"/>
+      <c r="BQ20" t="inlineStr"/>
+      <c r="BR20" t="inlineStr"/>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5849,6 +6089,16 @@
       <c r="BI21" t="inlineStr"/>
       <c r="BJ21" t="inlineStr"/>
       <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr"/>
+      <c r="BQ21" t="inlineStr"/>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6008,6 +6258,16 @@
       <c r="BI22" t="inlineStr"/>
       <c r="BJ22" t="inlineStr"/>
       <c r="BK22" t="inlineStr"/>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
+      <c r="BO22" t="inlineStr"/>
+      <c r="BP22" t="inlineStr"/>
+      <c r="BQ22" t="inlineStr"/>
+      <c r="BR22" t="inlineStr"/>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6167,6 +6427,16 @@
       <c r="BI23" t="inlineStr"/>
       <c r="BJ23" t="inlineStr"/>
       <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
+      <c r="BQ23" t="inlineStr"/>
+      <c r="BR23" t="inlineStr"/>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6326,6 +6596,16 @@
       <c r="BI24" t="inlineStr"/>
       <c r="BJ24" t="inlineStr"/>
       <c r="BK24" t="inlineStr"/>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
+      <c r="BO24" t="inlineStr"/>
+      <c r="BP24" t="inlineStr"/>
+      <c r="BQ24" t="inlineStr"/>
+      <c r="BR24" t="inlineStr"/>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6491,6 +6771,16 @@
       <c r="BI25" t="inlineStr"/>
       <c r="BJ25" t="inlineStr"/>
       <c r="BK25" t="inlineStr"/>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
+      <c r="BO25" t="inlineStr"/>
+      <c r="BP25" t="inlineStr"/>
+      <c r="BQ25" t="inlineStr"/>
+      <c r="BR25" t="inlineStr"/>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6656,6 +6946,16 @@
       <c r="BI26" t="inlineStr"/>
       <c r="BJ26" t="inlineStr"/>
       <c r="BK26" t="inlineStr"/>
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="inlineStr"/>
+      <c r="BN26" t="inlineStr"/>
+      <c r="BO26" t="inlineStr"/>
+      <c r="BP26" t="inlineStr"/>
+      <c r="BQ26" t="inlineStr"/>
+      <c r="BR26" t="inlineStr"/>
+      <c r="BS26" t="inlineStr"/>
+      <c r="BT26" t="inlineStr"/>
+      <c r="BU26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6821,6 +7121,16 @@
       <c r="BI27" t="inlineStr"/>
       <c r="BJ27" t="inlineStr"/>
       <c r="BK27" t="inlineStr"/>
+      <c r="BL27" t="inlineStr"/>
+      <c r="BM27" t="inlineStr"/>
+      <c r="BN27" t="inlineStr"/>
+      <c r="BO27" t="inlineStr"/>
+      <c r="BP27" t="inlineStr"/>
+      <c r="BQ27" t="inlineStr"/>
+      <c r="BR27" t="inlineStr"/>
+      <c r="BS27" t="inlineStr"/>
+      <c r="BT27" t="inlineStr"/>
+      <c r="BU27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6986,6 +7296,16 @@
       <c r="BI28" t="inlineStr"/>
       <c r="BJ28" t="inlineStr"/>
       <c r="BK28" t="inlineStr"/>
+      <c r="BL28" t="inlineStr"/>
+      <c r="BM28" t="inlineStr"/>
+      <c r="BN28" t="inlineStr"/>
+      <c r="BO28" t="inlineStr"/>
+      <c r="BP28" t="inlineStr"/>
+      <c r="BQ28" t="inlineStr"/>
+      <c r="BR28" t="inlineStr"/>
+      <c r="BS28" t="inlineStr"/>
+      <c r="BT28" t="inlineStr"/>
+      <c r="BU28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7151,6 +7471,16 @@
       <c r="BI29" t="inlineStr"/>
       <c r="BJ29" t="inlineStr"/>
       <c r="BK29" t="inlineStr"/>
+      <c r="BL29" t="inlineStr"/>
+      <c r="BM29" t="inlineStr"/>
+      <c r="BN29" t="inlineStr"/>
+      <c r="BO29" t="inlineStr"/>
+      <c r="BP29" t="inlineStr"/>
+      <c r="BQ29" t="inlineStr"/>
+      <c r="BR29" t="inlineStr"/>
+      <c r="BS29" t="inlineStr"/>
+      <c r="BT29" t="inlineStr"/>
+      <c r="BU29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7316,6 +7646,16 @@
       <c r="BI30" t="inlineStr"/>
       <c r="BJ30" t="inlineStr"/>
       <c r="BK30" t="inlineStr"/>
+      <c r="BL30" t="inlineStr"/>
+      <c r="BM30" t="inlineStr"/>
+      <c r="BN30" t="inlineStr"/>
+      <c r="BO30" t="inlineStr"/>
+      <c r="BP30" t="inlineStr"/>
+      <c r="BQ30" t="inlineStr"/>
+      <c r="BR30" t="inlineStr"/>
+      <c r="BS30" t="inlineStr"/>
+      <c r="BT30" t="inlineStr"/>
+      <c r="BU30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7481,6 +7821,16 @@
       <c r="BI31" t="inlineStr"/>
       <c r="BJ31" t="inlineStr"/>
       <c r="BK31" t="inlineStr"/>
+      <c r="BL31" t="inlineStr"/>
+      <c r="BM31" t="inlineStr"/>
+      <c r="BN31" t="inlineStr"/>
+      <c r="BO31" t="inlineStr"/>
+      <c r="BP31" t="inlineStr"/>
+      <c r="BQ31" t="inlineStr"/>
+      <c r="BR31" t="inlineStr"/>
+      <c r="BS31" t="inlineStr"/>
+      <c r="BT31" t="inlineStr"/>
+      <c r="BU31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7646,6 +7996,16 @@
       <c r="BI32" t="inlineStr"/>
       <c r="BJ32" t="inlineStr"/>
       <c r="BK32" t="inlineStr"/>
+      <c r="BL32" t="inlineStr"/>
+      <c r="BM32" t="inlineStr"/>
+      <c r="BN32" t="inlineStr"/>
+      <c r="BO32" t="inlineStr"/>
+      <c r="BP32" t="inlineStr"/>
+      <c r="BQ32" t="inlineStr"/>
+      <c r="BR32" t="inlineStr"/>
+      <c r="BS32" t="inlineStr"/>
+      <c r="BT32" t="inlineStr"/>
+      <c r="BU32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7813,6 +8173,16 @@
       <c r="BI33" t="inlineStr"/>
       <c r="BJ33" t="inlineStr"/>
       <c r="BK33" t="inlineStr"/>
+      <c r="BL33" t="inlineStr"/>
+      <c r="BM33" t="inlineStr"/>
+      <c r="BN33" t="inlineStr"/>
+      <c r="BO33" t="inlineStr"/>
+      <c r="BP33" t="inlineStr"/>
+      <c r="BQ33" t="inlineStr"/>
+      <c r="BR33" t="inlineStr"/>
+      <c r="BS33" t="inlineStr"/>
+      <c r="BT33" t="inlineStr"/>
+      <c r="BU33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7970,6 +8340,16 @@
       <c r="BI34" t="inlineStr"/>
       <c r="BJ34" t="inlineStr"/>
       <c r="BK34" t="inlineStr"/>
+      <c r="BL34" t="inlineStr"/>
+      <c r="BM34" t="inlineStr"/>
+      <c r="BN34" t="inlineStr"/>
+      <c r="BO34" t="inlineStr"/>
+      <c r="BP34" t="inlineStr"/>
+      <c r="BQ34" t="inlineStr"/>
+      <c r="BR34" t="inlineStr"/>
+      <c r="BS34" t="inlineStr"/>
+      <c r="BT34" t="inlineStr"/>
+      <c r="BU34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8143,6 +8523,16 @@
       <c r="BI35" t="inlineStr"/>
       <c r="BJ35" t="inlineStr"/>
       <c r="BK35" t="inlineStr"/>
+      <c r="BL35" t="inlineStr"/>
+      <c r="BM35" t="inlineStr"/>
+      <c r="BN35" t="inlineStr"/>
+      <c r="BO35" t="inlineStr"/>
+      <c r="BP35" t="inlineStr"/>
+      <c r="BQ35" t="inlineStr"/>
+      <c r="BR35" t="inlineStr"/>
+      <c r="BS35" t="inlineStr"/>
+      <c r="BT35" t="inlineStr"/>
+      <c r="BU35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8316,6 +8706,16 @@
       <c r="BI36" t="inlineStr"/>
       <c r="BJ36" t="inlineStr"/>
       <c r="BK36" t="inlineStr"/>
+      <c r="BL36" t="inlineStr"/>
+      <c r="BM36" t="inlineStr"/>
+      <c r="BN36" t="inlineStr"/>
+      <c r="BO36" t="inlineStr"/>
+      <c r="BP36" t="inlineStr"/>
+      <c r="BQ36" t="inlineStr"/>
+      <c r="BR36" t="inlineStr"/>
+      <c r="BS36" t="inlineStr"/>
+      <c r="BT36" t="inlineStr"/>
+      <c r="BU36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8489,6 +8889,16 @@
       <c r="BI37" t="inlineStr"/>
       <c r="BJ37" t="inlineStr"/>
       <c r="BK37" t="inlineStr"/>
+      <c r="BL37" t="inlineStr"/>
+      <c r="BM37" t="inlineStr"/>
+      <c r="BN37" t="inlineStr"/>
+      <c r="BO37" t="inlineStr"/>
+      <c r="BP37" t="inlineStr"/>
+      <c r="BQ37" t="inlineStr"/>
+      <c r="BR37" t="inlineStr"/>
+      <c r="BS37" t="inlineStr"/>
+      <c r="BT37" t="inlineStr"/>
+      <c r="BU37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8682,6 +9092,16 @@
       <c r="BI38" t="inlineStr"/>
       <c r="BJ38" t="inlineStr"/>
       <c r="BK38" t="inlineStr"/>
+      <c r="BL38" t="inlineStr"/>
+      <c r="BM38" t="inlineStr"/>
+      <c r="BN38" t="inlineStr"/>
+      <c r="BO38" t="inlineStr"/>
+      <c r="BP38" t="inlineStr"/>
+      <c r="BQ38" t="inlineStr"/>
+      <c r="BR38" t="inlineStr"/>
+      <c r="BS38" t="inlineStr"/>
+      <c r="BT38" t="inlineStr"/>
+      <c r="BU38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8875,6 +9295,16 @@
       <c r="BI39" t="inlineStr"/>
       <c r="BJ39" t="inlineStr"/>
       <c r="BK39" t="inlineStr"/>
+      <c r="BL39" t="inlineStr"/>
+      <c r="BM39" t="inlineStr"/>
+      <c r="BN39" t="inlineStr"/>
+      <c r="BO39" t="inlineStr"/>
+      <c r="BP39" t="inlineStr"/>
+      <c r="BQ39" t="inlineStr"/>
+      <c r="BR39" t="inlineStr"/>
+      <c r="BS39" t="inlineStr"/>
+      <c r="BT39" t="inlineStr"/>
+      <c r="BU39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9070,6 +9500,16 @@
       <c r="BI40" t="inlineStr"/>
       <c r="BJ40" t="inlineStr"/>
       <c r="BK40" t="inlineStr"/>
+      <c r="BL40" t="inlineStr"/>
+      <c r="BM40" t="inlineStr"/>
+      <c r="BN40" t="inlineStr"/>
+      <c r="BO40" t="inlineStr"/>
+      <c r="BP40" t="inlineStr"/>
+      <c r="BQ40" t="inlineStr"/>
+      <c r="BR40" t="inlineStr"/>
+      <c r="BS40" t="inlineStr"/>
+      <c r="BT40" t="inlineStr"/>
+      <c r="BU40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9267,6 +9707,16 @@
       </c>
       <c r="BJ41" t="inlineStr"/>
       <c r="BK41" t="inlineStr"/>
+      <c r="BL41" t="inlineStr"/>
+      <c r="BM41" t="inlineStr"/>
+      <c r="BN41" t="inlineStr"/>
+      <c r="BO41" t="inlineStr"/>
+      <c r="BP41" t="inlineStr"/>
+      <c r="BQ41" t="inlineStr"/>
+      <c r="BR41" t="inlineStr"/>
+      <c r="BS41" t="inlineStr"/>
+      <c r="BT41" t="inlineStr"/>
+      <c r="BU41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9464,6 +9914,16 @@
       </c>
       <c r="BJ42" t="inlineStr"/>
       <c r="BK42" t="inlineStr"/>
+      <c r="BL42" t="inlineStr"/>
+      <c r="BM42" t="inlineStr"/>
+      <c r="BN42" t="inlineStr"/>
+      <c r="BO42" t="inlineStr"/>
+      <c r="BP42" t="inlineStr"/>
+      <c r="BQ42" t="inlineStr"/>
+      <c r="BR42" t="inlineStr"/>
+      <c r="BS42" t="inlineStr"/>
+      <c r="BT42" t="inlineStr"/>
+      <c r="BU42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9661,6 +10121,16 @@
       </c>
       <c r="BJ43" t="inlineStr"/>
       <c r="BK43" t="inlineStr"/>
+      <c r="BL43" t="inlineStr"/>
+      <c r="BM43" t="inlineStr"/>
+      <c r="BN43" t="inlineStr"/>
+      <c r="BO43" t="inlineStr"/>
+      <c r="BP43" t="inlineStr"/>
+      <c r="BQ43" t="inlineStr"/>
+      <c r="BR43" t="inlineStr"/>
+      <c r="BS43" t="inlineStr"/>
+      <c r="BT43" t="inlineStr"/>
+      <c r="BU43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9858,6 +10328,16 @@
       </c>
       <c r="BJ44" t="inlineStr"/>
       <c r="BK44" t="inlineStr"/>
+      <c r="BL44" t="inlineStr"/>
+      <c r="BM44" t="inlineStr"/>
+      <c r="BN44" t="inlineStr"/>
+      <c r="BO44" t="inlineStr"/>
+      <c r="BP44" t="inlineStr"/>
+      <c r="BQ44" t="inlineStr"/>
+      <c r="BR44" t="inlineStr"/>
+      <c r="BS44" t="inlineStr"/>
+      <c r="BT44" t="inlineStr"/>
+      <c r="BU44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10057,6 +10537,16 @@
         <v>1</v>
       </c>
       <c r="BK45" t="inlineStr"/>
+      <c r="BL45" t="inlineStr"/>
+      <c r="BM45" t="inlineStr"/>
+      <c r="BN45" t="inlineStr"/>
+      <c r="BO45" t="inlineStr"/>
+      <c r="BP45" t="inlineStr"/>
+      <c r="BQ45" t="inlineStr"/>
+      <c r="BR45" t="inlineStr"/>
+      <c r="BS45" t="inlineStr"/>
+      <c r="BT45" t="inlineStr"/>
+      <c r="BU45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10256,6 +10746,16 @@
         <v>1</v>
       </c>
       <c r="BK46" t="inlineStr"/>
+      <c r="BL46" t="inlineStr"/>
+      <c r="BM46" t="inlineStr"/>
+      <c r="BN46" t="inlineStr"/>
+      <c r="BO46" t="inlineStr"/>
+      <c r="BP46" t="inlineStr"/>
+      <c r="BQ46" t="inlineStr"/>
+      <c r="BR46" t="inlineStr"/>
+      <c r="BS46" t="inlineStr"/>
+      <c r="BT46" t="inlineStr"/>
+      <c r="BU46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10457,6 +10957,16 @@
       <c r="BK47" t="n">
         <v>2</v>
       </c>
+      <c r="BL47" t="inlineStr"/>
+      <c r="BM47" t="inlineStr"/>
+      <c r="BN47" t="inlineStr"/>
+      <c r="BO47" t="inlineStr"/>
+      <c r="BP47" t="inlineStr"/>
+      <c r="BQ47" t="inlineStr"/>
+      <c r="BR47" t="inlineStr"/>
+      <c r="BS47" t="inlineStr"/>
+      <c r="BT47" t="inlineStr"/>
+      <c r="BU47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10658,6 +11168,16 @@
       <c r="BK48" t="n">
         <v>2</v>
       </c>
+      <c r="BL48" t="inlineStr"/>
+      <c r="BM48" t="inlineStr"/>
+      <c r="BN48" t="inlineStr"/>
+      <c r="BO48" t="inlineStr"/>
+      <c r="BP48" t="inlineStr"/>
+      <c r="BQ48" t="inlineStr"/>
+      <c r="BR48" t="inlineStr"/>
+      <c r="BS48" t="inlineStr"/>
+      <c r="BT48" t="inlineStr"/>
+      <c r="BU48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -10859,6 +11379,16 @@
       <c r="BK49" t="n">
         <v>2</v>
       </c>
+      <c r="BL49" t="inlineStr"/>
+      <c r="BM49" t="inlineStr"/>
+      <c r="BN49" t="inlineStr"/>
+      <c r="BO49" t="inlineStr"/>
+      <c r="BP49" t="inlineStr"/>
+      <c r="BQ49" t="inlineStr"/>
+      <c r="BR49" t="inlineStr"/>
+      <c r="BS49" t="inlineStr"/>
+      <c r="BT49" t="inlineStr"/>
+      <c r="BU49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11059,6 +11589,1414 @@
       </c>
       <c r="BK50" t="n">
         <v>2</v>
+      </c>
+      <c r="BL50" t="inlineStr"/>
+      <c r="BM50" t="inlineStr"/>
+      <c r="BN50" t="inlineStr"/>
+      <c r="BO50" t="inlineStr"/>
+      <c r="BP50" t="inlineStr"/>
+      <c r="BQ50" t="inlineStr"/>
+      <c r="BR50" t="inlineStr"/>
+      <c r="BS50" t="inlineStr"/>
+      <c r="BT50" t="inlineStr"/>
+      <c r="BU50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_full_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>47</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G51" t="n">
+        <v>100</v>
+      </c>
+      <c r="H51" t="n">
+        <v>100</v>
+      </c>
+      <c r="I51" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L51" t="n">
+        <v>24</v>
+      </c>
+      <c r="M51" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S51" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U51" t="n">
+        <v>33.24460387229919</v>
+      </c>
+      <c r="V51" t="n">
+        <v>0.8911775512134743</v>
+      </c>
+      <c r="W51" t="n">
+        <v>2</v>
+      </c>
+      <c r="X51" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0.1294373368094012</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>8.695240541449178e-05</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG51" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH51" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK51" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP51" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR51" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT51" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV51" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA51" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB51" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC51" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD51" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE51" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF51" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG51" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ51" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK51" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN51" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO51" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP51" t="n">
+        <v>0.5041189721373261</v>
+      </c>
+      <c r="BQ51" t="n">
+        <v>0.004516136714211497</v>
+      </c>
+      <c r="BR51" t="n">
+        <v>0.5141972166592957</v>
+      </c>
+      <c r="BS51" t="n">
+        <v>0.5063661898745865</v>
+      </c>
+      <c r="BT51" t="n">
+        <v>0.0001869450772246041</v>
+      </c>
+      <c r="BU51" t="n">
+        <v>0.1304726324609068</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_holddelta_nas100_seed47_cuda</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>47</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G52" t="n">
+        <v>100</v>
+      </c>
+      <c r="H52" t="n">
+        <v>100</v>
+      </c>
+      <c r="I52" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L52" t="n">
+        <v>24</v>
+      </c>
+      <c r="M52" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S52" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U52" t="n">
+        <v>35.00389361381531</v>
+      </c>
+      <c r="V52" t="n">
+        <v>0.8911775512134743</v>
+      </c>
+      <c r="W52" t="n">
+        <v>2</v>
+      </c>
+      <c r="X52" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>0.1165822199419366</v>
+      </c>
+      <c r="AA52" t="n">
+        <v>6.578008647846553e-05</v>
+      </c>
+      <c r="AB52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD52" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE52" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF52" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH52" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ52" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK52" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP52" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR52" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS52" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV52" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA52" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB52" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC52" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD52" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE52" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF52" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG52" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ52" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK52" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM52" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN52" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO52" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP52" t="n">
+        <v>0.5015627399819796</v>
+      </c>
+      <c r="BQ52" t="n">
+        <v>0.004526531569980329</v>
+      </c>
+      <c r="BR52" t="n">
+        <v>0.5116963352336258</v>
+      </c>
+      <c r="BS52" t="n">
+        <v>0.5038472748682147</v>
+      </c>
+      <c r="BT52" t="n">
+        <v>0.0001884428960782644</v>
+      </c>
+      <c r="BU52" t="n">
+        <v>0.1304918363934658</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_full_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>77</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G53" t="n">
+        <v>100</v>
+      </c>
+      <c r="H53" t="n">
+        <v>100</v>
+      </c>
+      <c r="I53" t="n">
+        <v>2.539606015961426</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.3934536132812501</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.1204159526154336</v>
+      </c>
+      <c r="L53" t="n">
+        <v>5</v>
+      </c>
+      <c r="M53" t="n">
+        <v>19.33333333333333</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="n">
+        <v>8.766938595101237</v>
+      </c>
+      <c r="S53" t="n">
+        <v>0.5386988712707534</v>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U53" t="n">
+        <v>34.08843159675598</v>
+      </c>
+      <c r="V53" t="n">
+        <v>2.539606015961426</v>
+      </c>
+      <c r="W53" t="n">
+        <v>0</v>
+      </c>
+      <c r="X53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>0.3583201341575816</v>
+      </c>
+      <c r="AA53" t="n">
+        <v>3.513544212789081e-05</v>
+      </c>
+      <c r="AB53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD53" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE53" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF53" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG53" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH53" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="AI53" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AJ53" t="n">
+        <v>21</v>
+      </c>
+      <c r="AK53" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR53" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT53" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU53" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV53" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA53" t="n">
+        <v>0.0002132128484563196</v>
+      </c>
+      <c r="BB53" t="n">
+        <v>0.006864221211611132</v>
+      </c>
+      <c r="BC53" t="n">
+        <v>0.5172413793103449</v>
+      </c>
+      <c r="BD53" t="n">
+        <v>-0.0001604645442747479</v>
+      </c>
+      <c r="BE53" t="n">
+        <v>0.4913793103448276</v>
+      </c>
+      <c r="BF53" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BG53" t="n">
+        <v>0.4864864864864865</v>
+      </c>
+      <c r="BH53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ53" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK53" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM53" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN53" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO53" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP53" t="n">
+        <v>0.5011665661787165</v>
+      </c>
+      <c r="BQ53" t="n">
+        <v>0.005072661446696469</v>
+      </c>
+      <c r="BR53" t="n">
+        <v>0.5128883436836046</v>
+      </c>
+      <c r="BS53" t="n">
+        <v>0.5051945715114988</v>
+      </c>
+      <c r="BT53" t="n">
+        <v>0.001970421281996472</v>
+      </c>
+      <c r="BU53" t="n">
+        <v>0.0962601557117084</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_holddelta_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>77</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G54" t="n">
+        <v>100</v>
+      </c>
+      <c r="H54" t="n">
+        <v>100</v>
+      </c>
+      <c r="I54" t="n">
+        <v>2.852980205253647</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.429462890625</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.1270832360013094</v>
+      </c>
+      <c r="L54" t="n">
+        <v>5</v>
+      </c>
+      <c r="M54" t="n">
+        <v>19.33333333333333</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="n">
+        <v>9.055825112387538</v>
+      </c>
+      <c r="S54" t="n">
+        <v>0.5791051973064896</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U54" t="n">
+        <v>33.7391562461853</v>
+      </c>
+      <c r="V54" t="n">
+        <v>2.852980205253647</v>
+      </c>
+      <c r="W54" t="n">
+        <v>0</v>
+      </c>
+      <c r="X54" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>0.3680209930522198</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>3.448805554875262e-05</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE54" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG54" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH54" t="n">
+        <v>23</v>
+      </c>
+      <c r="AI54" t="n">
+        <v>0.8944271909999159</v>
+      </c>
+      <c r="AJ54" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK54" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR54" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA54" t="n">
+        <v>-0.0002687426538864986</v>
+      </c>
+      <c r="BB54" t="n">
+        <v>0.006335475392727952</v>
+      </c>
+      <c r="BC54" t="n">
+        <v>0.456896551724138</v>
+      </c>
+      <c r="BD54" t="n">
+        <v>-0.0002131501889129266</v>
+      </c>
+      <c r="BE54" t="n">
+        <v>0.5344827586206896</v>
+      </c>
+      <c r="BF54" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BG54" t="n">
+        <v>0.5405405405405406</v>
+      </c>
+      <c r="BH54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ54" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK54" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM54" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN54" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO54" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP54" t="n">
+        <v>0.5008735029861845</v>
+      </c>
+      <c r="BQ54" t="n">
+        <v>0.004878828534856439</v>
+      </c>
+      <c r="BR54" t="n">
+        <v>0.5114729091011244</v>
+      </c>
+      <c r="BS54" t="n">
+        <v>0.5049401943025917</v>
+      </c>
+      <c r="BT54" t="n">
+        <v>0.001542419949867602</v>
+      </c>
+      <c r="BU54" t="n">
+        <v>0.09612672339225638</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_delta_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>77</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>5</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G55" t="n">
+        <v>100</v>
+      </c>
+      <c r="H55" t="n">
+        <v>100</v>
+      </c>
+      <c r="I55" t="n">
+        <v>2.421347629868198</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.3543841552734375</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.1410848734196286</v>
+      </c>
+      <c r="L55" t="n">
+        <v>4</v>
+      </c>
+      <c r="M55" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" t="n">
+        <v>8.606393596157432</v>
+      </c>
+      <c r="S55" t="n">
+        <v>0.5164769915572833</v>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U55" t="n">
+        <v>53.12738656997681</v>
+      </c>
+      <c r="V55" t="n">
+        <v>2.421347629868198</v>
+      </c>
+      <c r="W55" t="n">
+        <v>0</v>
+      </c>
+      <c r="X55" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>0.3498953277062355</v>
+      </c>
+      <c r="AA55" t="n">
+        <v>2.99935594133179e-05</v>
+      </c>
+      <c r="AB55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD55" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE55" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF55" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG55" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH55" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="AI55" t="n">
+        <v>0.4330127018922193</v>
+      </c>
+      <c r="AJ55" t="n">
+        <v>23</v>
+      </c>
+      <c r="AK55" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR55" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS55" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT55" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU55" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV55" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA55" t="n">
+        <v>0.0003852021071562094</v>
+      </c>
+      <c r="BB55" t="n">
+        <v>0.007053353232612577</v>
+      </c>
+      <c r="BC55" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD55" t="n">
+        <v>-0.000251485453316428</v>
+      </c>
+      <c r="BE55" t="n">
+        <v>0.5344827586206896</v>
+      </c>
+      <c r="BF55" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BG55" t="n">
+        <v>0.5357142857142857</v>
+      </c>
+      <c r="BH55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ55" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK55" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM55" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN55" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO55" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="BP55" t="n">
+        <v>0.5023902428561243</v>
+      </c>
+      <c r="BQ55" t="n">
+        <v>0.005028468556702137</v>
+      </c>
+      <c r="BR55" t="n">
+        <v>0.5133042484521866</v>
+      </c>
+      <c r="BS55" t="n">
+        <v>0.5065005164721916</v>
+      </c>
+      <c r="BT55" t="n">
+        <v>0.001809040110574329</v>
+      </c>
+      <c r="BU55" t="n">
+        <v>0.09616787262774747</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>pg_smoke_gate_holddelta_nas100_seed47_boundary10_cuda</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>47</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>8</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G56" t="n">
+        <v>100</v>
+      </c>
+      <c r="H56" t="n">
+        <v>100</v>
+      </c>
+      <c r="I56" t="n">
+        <v>3.285968442308683</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.2795610351562501</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.07478926481247072</v>
+      </c>
+      <c r="L56" t="n">
+        <v>2</v>
+      </c>
+      <c r="M56" t="n">
+        <v>40.66666666666666</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" t="n">
+        <v>4.930687682703137</v>
+      </c>
+      <c r="S56" t="n">
+        <v>0.2960980424541049</v>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U56" t="n">
+        <v>77.07337546348572</v>
+      </c>
+      <c r="V56" t="n">
+        <v>3.285968442308683</v>
+      </c>
+      <c r="W56" t="n">
+        <v>0</v>
+      </c>
+      <c r="X56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y56" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>0.4104356466205736</v>
+      </c>
+      <c r="AA56" t="n">
+        <v>3.765037091887699e-05</v>
+      </c>
+      <c r="AB56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD56" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE56" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF56" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG56" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH56" t="n">
+        <v>42</v>
+      </c>
+      <c r="AI56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ56" t="n">
+        <v>42</v>
+      </c>
+      <c r="AK56" t="n">
+        <v>42</v>
+      </c>
+      <c r="AL56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR56" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS56" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT56" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU56" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV56" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW56" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX56" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA56" t="n">
+        <v>-6.822393259456281e-05</v>
+      </c>
+      <c r="BB56" t="n">
+        <v>0.003457659564953589</v>
+      </c>
+      <c r="BC56" t="n">
+        <v>0.4180327868852459</v>
+      </c>
+      <c r="BD56" t="n">
+        <v>0.0001877821474915779</v>
+      </c>
+      <c r="BE56" t="n">
+        <v>0.5819672131147541</v>
+      </c>
+      <c r="BF56" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BG56" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="BH56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ56" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK56" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL56" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM56" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN56" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO56" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP56" t="n">
+        <v>0.5033096216741155</v>
+      </c>
+      <c r="BQ56" t="n">
+        <v>0.004051795277026956</v>
+      </c>
+      <c r="BR56" t="n">
+        <v>0.5130154148477023</v>
+      </c>
+      <c r="BS56" t="n">
+        <v>0.5048100542826731</v>
+      </c>
+      <c r="BT56" t="n">
+        <v>0.001163482550554527</v>
+      </c>
+      <c r="BU56" t="n">
+        <v>0.1303519422157866</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add hold biased PG controller initialization
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2980,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BU56"/>
+  <dimension ref="A1:BW68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3347,6 +3347,16 @@
       <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>gate_top5_mass</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>initial_hold_bias</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>zero_policy_output</t>
         </is>
       </c>
     </row>
@@ -3474,6 +3484,8 @@
       <c r="BS2" t="inlineStr"/>
       <c r="BT2" t="inlineStr"/>
       <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3599,6 +3611,8 @@
       <c r="BS3" t="inlineStr"/>
       <c r="BT3" t="inlineStr"/>
       <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr"/>
+      <c r="BW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3724,6 +3738,8 @@
       <c r="BS4" t="inlineStr"/>
       <c r="BT4" t="inlineStr"/>
       <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3849,6 +3865,8 @@
       <c r="BS5" t="inlineStr"/>
       <c r="BT5" t="inlineStr"/>
       <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr"/>
+      <c r="BW5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3978,6 +3996,8 @@
       <c r="BS6" t="inlineStr"/>
       <c r="BT6" t="inlineStr"/>
       <c r="BU6" t="inlineStr"/>
+      <c r="BV6" t="inlineStr"/>
+      <c r="BW6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4107,6 +4127,8 @@
       <c r="BS7" t="inlineStr"/>
       <c r="BT7" t="inlineStr"/>
       <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr"/>
+      <c r="BW7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4238,6 +4260,8 @@
       <c r="BS8" t="inlineStr"/>
       <c r="BT8" t="inlineStr"/>
       <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4369,6 +4393,8 @@
       <c r="BS9" t="inlineStr"/>
       <c r="BT9" t="inlineStr"/>
       <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4502,6 +4528,8 @@
       <c r="BS10" t="inlineStr"/>
       <c r="BT10" t="inlineStr"/>
       <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4643,6 +4671,8 @@
       <c r="BS11" t="inlineStr"/>
       <c r="BT11" t="inlineStr"/>
       <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4784,6 +4814,8 @@
       <c r="BS12" t="inlineStr"/>
       <c r="BT12" t="inlineStr"/>
       <c r="BU12" t="inlineStr"/>
+      <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4927,6 +4959,8 @@
       <c r="BS13" t="inlineStr"/>
       <c r="BT13" t="inlineStr"/>
       <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5070,6 +5104,8 @@
       <c r="BS14" t="inlineStr"/>
       <c r="BT14" t="inlineStr"/>
       <c r="BU14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5217,6 +5253,8 @@
       <c r="BS15" t="inlineStr"/>
       <c r="BT15" t="inlineStr"/>
       <c r="BU15" t="inlineStr"/>
+      <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5364,6 +5402,8 @@
       <c r="BS16" t="inlineStr"/>
       <c r="BT16" t="inlineStr"/>
       <c r="BU16" t="inlineStr"/>
+      <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5511,6 +5551,8 @@
       <c r="BS17" t="inlineStr"/>
       <c r="BT17" t="inlineStr"/>
       <c r="BU17" t="inlineStr"/>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5658,6 +5700,8 @@
       <c r="BS18" t="inlineStr"/>
       <c r="BT18" t="inlineStr"/>
       <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5805,6 +5849,8 @@
       <c r="BS19" t="inlineStr"/>
       <c r="BT19" t="inlineStr"/>
       <c r="BU19" t="inlineStr"/>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5952,6 +5998,8 @@
       <c r="BS20" t="inlineStr"/>
       <c r="BT20" t="inlineStr"/>
       <c r="BU20" t="inlineStr"/>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6099,6 +6147,8 @@
       <c r="BS21" t="inlineStr"/>
       <c r="BT21" t="inlineStr"/>
       <c r="BU21" t="inlineStr"/>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6268,6 +6318,8 @@
       <c r="BS22" t="inlineStr"/>
       <c r="BT22" t="inlineStr"/>
       <c r="BU22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr"/>
+      <c r="BW22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6437,6 +6489,8 @@
       <c r="BS23" t="inlineStr"/>
       <c r="BT23" t="inlineStr"/>
       <c r="BU23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr"/>
+      <c r="BW23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6606,6 +6660,8 @@
       <c r="BS24" t="inlineStr"/>
       <c r="BT24" t="inlineStr"/>
       <c r="BU24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr"/>
+      <c r="BW24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6781,6 +6837,8 @@
       <c r="BS25" t="inlineStr"/>
       <c r="BT25" t="inlineStr"/>
       <c r="BU25" t="inlineStr"/>
+      <c r="BV25" t="inlineStr"/>
+      <c r="BW25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6956,6 +7014,8 @@
       <c r="BS26" t="inlineStr"/>
       <c r="BT26" t="inlineStr"/>
       <c r="BU26" t="inlineStr"/>
+      <c r="BV26" t="inlineStr"/>
+      <c r="BW26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7131,6 +7191,8 @@
       <c r="BS27" t="inlineStr"/>
       <c r="BT27" t="inlineStr"/>
       <c r="BU27" t="inlineStr"/>
+      <c r="BV27" t="inlineStr"/>
+      <c r="BW27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7306,6 +7368,8 @@
       <c r="BS28" t="inlineStr"/>
       <c r="BT28" t="inlineStr"/>
       <c r="BU28" t="inlineStr"/>
+      <c r="BV28" t="inlineStr"/>
+      <c r="BW28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7481,6 +7545,8 @@
       <c r="BS29" t="inlineStr"/>
       <c r="BT29" t="inlineStr"/>
       <c r="BU29" t="inlineStr"/>
+      <c r="BV29" t="inlineStr"/>
+      <c r="BW29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7656,6 +7722,8 @@
       <c r="BS30" t="inlineStr"/>
       <c r="BT30" t="inlineStr"/>
       <c r="BU30" t="inlineStr"/>
+      <c r="BV30" t="inlineStr"/>
+      <c r="BW30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7831,6 +7899,8 @@
       <c r="BS31" t="inlineStr"/>
       <c r="BT31" t="inlineStr"/>
       <c r="BU31" t="inlineStr"/>
+      <c r="BV31" t="inlineStr"/>
+      <c r="BW31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8006,6 +8076,8 @@
       <c r="BS32" t="inlineStr"/>
       <c r="BT32" t="inlineStr"/>
       <c r="BU32" t="inlineStr"/>
+      <c r="BV32" t="inlineStr"/>
+      <c r="BW32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8183,6 +8255,8 @@
       <c r="BS33" t="inlineStr"/>
       <c r="BT33" t="inlineStr"/>
       <c r="BU33" t="inlineStr"/>
+      <c r="BV33" t="inlineStr"/>
+      <c r="BW33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8350,6 +8424,8 @@
       <c r="BS34" t="inlineStr"/>
       <c r="BT34" t="inlineStr"/>
       <c r="BU34" t="inlineStr"/>
+      <c r="BV34" t="inlineStr"/>
+      <c r="BW34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8533,6 +8609,8 @@
       <c r="BS35" t="inlineStr"/>
       <c r="BT35" t="inlineStr"/>
       <c r="BU35" t="inlineStr"/>
+      <c r="BV35" t="inlineStr"/>
+      <c r="BW35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8716,6 +8794,8 @@
       <c r="BS36" t="inlineStr"/>
       <c r="BT36" t="inlineStr"/>
       <c r="BU36" t="inlineStr"/>
+      <c r="BV36" t="inlineStr"/>
+      <c r="BW36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8899,6 +8979,8 @@
       <c r="BS37" t="inlineStr"/>
       <c r="BT37" t="inlineStr"/>
       <c r="BU37" t="inlineStr"/>
+      <c r="BV37" t="inlineStr"/>
+      <c r="BW37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9102,6 +9184,8 @@
       <c r="BS38" t="inlineStr"/>
       <c r="BT38" t="inlineStr"/>
       <c r="BU38" t="inlineStr"/>
+      <c r="BV38" t="inlineStr"/>
+      <c r="BW38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9305,6 +9389,8 @@
       <c r="BS39" t="inlineStr"/>
       <c r="BT39" t="inlineStr"/>
       <c r="BU39" t="inlineStr"/>
+      <c r="BV39" t="inlineStr"/>
+      <c r="BW39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -9510,6 +9596,8 @@
       <c r="BS40" t="inlineStr"/>
       <c r="BT40" t="inlineStr"/>
       <c r="BU40" t="inlineStr"/>
+      <c r="BV40" t="inlineStr"/>
+      <c r="BW40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9717,6 +9805,8 @@
       <c r="BS41" t="inlineStr"/>
       <c r="BT41" t="inlineStr"/>
       <c r="BU41" t="inlineStr"/>
+      <c r="BV41" t="inlineStr"/>
+      <c r="BW41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9924,6 +10014,8 @@
       <c r="BS42" t="inlineStr"/>
       <c r="BT42" t="inlineStr"/>
       <c r="BU42" t="inlineStr"/>
+      <c r="BV42" t="inlineStr"/>
+      <c r="BW42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -10131,6 +10223,8 @@
       <c r="BS43" t="inlineStr"/>
       <c r="BT43" t="inlineStr"/>
       <c r="BU43" t="inlineStr"/>
+      <c r="BV43" t="inlineStr"/>
+      <c r="BW43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -10338,6 +10432,8 @@
       <c r="BS44" t="inlineStr"/>
       <c r="BT44" t="inlineStr"/>
       <c r="BU44" t="inlineStr"/>
+      <c r="BV44" t="inlineStr"/>
+      <c r="BW44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -10547,6 +10643,8 @@
       <c r="BS45" t="inlineStr"/>
       <c r="BT45" t="inlineStr"/>
       <c r="BU45" t="inlineStr"/>
+      <c r="BV45" t="inlineStr"/>
+      <c r="BW45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -10756,6 +10854,8 @@
       <c r="BS46" t="inlineStr"/>
       <c r="BT46" t="inlineStr"/>
       <c r="BU46" t="inlineStr"/>
+      <c r="BV46" t="inlineStr"/>
+      <c r="BW46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -10967,6 +11067,8 @@
       <c r="BS47" t="inlineStr"/>
       <c r="BT47" t="inlineStr"/>
       <c r="BU47" t="inlineStr"/>
+      <c r="BV47" t="inlineStr"/>
+      <c r="BW47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -11178,6 +11280,8 @@
       <c r="BS48" t="inlineStr"/>
       <c r="BT48" t="inlineStr"/>
       <c r="BU48" t="inlineStr"/>
+      <c r="BV48" t="inlineStr"/>
+      <c r="BW48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -11389,6 +11493,8 @@
       <c r="BS49" t="inlineStr"/>
       <c r="BT49" t="inlineStr"/>
       <c r="BU49" t="inlineStr"/>
+      <c r="BV49" t="inlineStr"/>
+      <c r="BW49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -11600,6 +11706,8 @@
       <c r="BS50" t="inlineStr"/>
       <c r="BT50" t="inlineStr"/>
       <c r="BU50" t="inlineStr"/>
+      <c r="BV50" t="inlineStr"/>
+      <c r="BW50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -11833,6 +11941,8 @@
       <c r="BU51" t="n">
         <v>0.1304726324609068</v>
       </c>
+      <c r="BV51" t="inlineStr"/>
+      <c r="BW51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -12066,6 +12176,8 @@
       <c r="BU52" t="n">
         <v>0.1304918363934658</v>
       </c>
+      <c r="BV52" t="inlineStr"/>
+      <c r="BW52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -12299,6 +12411,8 @@
       <c r="BU53" t="n">
         <v>0.0962601557117084</v>
       </c>
+      <c r="BV53" t="inlineStr"/>
+      <c r="BW53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -12532,6 +12646,8 @@
       <c r="BU54" t="n">
         <v>0.09612672339225638</v>
       </c>
+      <c r="BV54" t="inlineStr"/>
+      <c r="BW54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -12765,6 +12881,8 @@
       <c r="BU55" t="n">
         <v>0.09616787262774747</v>
       </c>
+      <c r="BV55" t="inlineStr"/>
+      <c r="BW55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -12997,6 +13115,2852 @@
       </c>
       <c r="BU56" t="n">
         <v>0.1303519422157866</v>
+      </c>
+      <c r="BV56" t="inlineStr"/>
+      <c r="BW56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_sh_seed77_cuda</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>77</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>20</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G57" t="n">
+        <v>100</v>
+      </c>
+      <c r="H57" t="n">
+        <v>100</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.6146965283247042</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.2616151123046875</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.2450683373772208</v>
+      </c>
+      <c r="L57" t="n">
+        <v>21</v>
+      </c>
+      <c r="M57" t="n">
+        <v>22.04545454545455</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" t="n">
+        <v>42.20960809476674</v>
+      </c>
+      <c r="S57" t="n">
+        <v>2.123654276889283</v>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U57" t="n">
+        <v>1556.338429450989</v>
+      </c>
+      <c r="V57" t="n">
+        <v>0.6146965283247042</v>
+      </c>
+      <c r="W57" t="n">
+        <v>0</v>
+      </c>
+      <c r="X57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>0.3667019346382751</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>3.4746860150376e-05</v>
+      </c>
+      <c r="AB57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD57" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE57" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF57" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH57" t="n">
+        <v>22.85714285714286</v>
+      </c>
+      <c r="AI57" t="n">
+        <v>0.8883218145798872</v>
+      </c>
+      <c r="AJ57" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK57" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR57" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS57" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU57" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV57" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA57" t="n">
+        <v>-0.0004129861543295886</v>
+      </c>
+      <c r="BB57" t="n">
+        <v>0.006861430417671895</v>
+      </c>
+      <c r="BC57" t="n">
+        <v>0.4701030927835051</v>
+      </c>
+      <c r="BD57" t="n">
+        <v>0.0003100455704399567</v>
+      </c>
+      <c r="BE57" t="n">
+        <v>0.5237113402061856</v>
+      </c>
+      <c r="BF57" t="n">
+        <v>0.4285714285714285</v>
+      </c>
+      <c r="BG57" t="n">
+        <v>0.5280172413793104</v>
+      </c>
+      <c r="BH57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ57" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK57" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM57" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN57" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO57" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP57" t="n">
+        <v>0.5004961078314437</v>
+      </c>
+      <c r="BQ57" t="n">
+        <v>0.005283040086709961</v>
+      </c>
+      <c r="BR57" t="n">
+        <v>0.5124819351225784</v>
+      </c>
+      <c r="BS57" t="n">
+        <v>0.5053118290974922</v>
+      </c>
+      <c r="BT57" t="n">
+        <v>0.0006563626128949763</v>
+      </c>
+      <c r="BU57" t="n">
+        <v>0.09632927382115236</v>
+      </c>
+      <c r="BV57" t="inlineStr"/>
+      <c r="BW57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_nas100_seed47_boundary10_cuda</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>47</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>20</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G58" t="n">
+        <v>100</v>
+      </c>
+      <c r="H58" t="n">
+        <v>100</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.7239505399598438</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.4715556640625</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.3736568652803145</v>
+      </c>
+      <c r="L58" t="n">
+        <v>42</v>
+      </c>
+      <c r="M58" t="n">
+        <v>13.44186046511628</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" t="n">
+        <v>52.66407420299947</v>
+      </c>
+      <c r="S58" t="n">
+        <v>3.394109065004159</v>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U58" t="n">
+        <v>1575.273771286011</v>
+      </c>
+      <c r="V58" t="n">
+        <v>0.009664825674129629</v>
+      </c>
+      <c r="W58" t="n">
+        <v>0.7142857142857142</v>
+      </c>
+      <c r="X58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>0.3470945350463902</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>4.403810309541282e-05</v>
+      </c>
+      <c r="AB58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD58" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE58" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF58" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG58" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH58" t="n">
+        <v>13.66666666666667</v>
+      </c>
+      <c r="AI58" t="n">
+        <v>8.481539243351289</v>
+      </c>
+      <c r="AJ58" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK58" t="n">
+        <v>34</v>
+      </c>
+      <c r="AL58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP58" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ58" t="n">
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="AR58" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT58" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU58" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV58" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA58" t="n">
+        <v>6.183299337611227e-05</v>
+      </c>
+      <c r="BB58" t="n">
+        <v>0.004022203314455047</v>
+      </c>
+      <c r="BC58" t="n">
+        <v>0.4705882352941176</v>
+      </c>
+      <c r="BD58" t="n">
+        <v>-0.000170529264761143</v>
+      </c>
+      <c r="BE58" t="n">
+        <v>0.5259515570934256</v>
+      </c>
+      <c r="BF58" t="n">
+        <v>0.4761904761904762</v>
+      </c>
+      <c r="BG58" t="n">
+        <v>0.5298507462686567</v>
+      </c>
+      <c r="BH58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ58" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK58" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL58" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM58" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN58" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO58" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP58" t="n">
+        <v>0.5009725921913002</v>
+      </c>
+      <c r="BQ58" t="n">
+        <v>0.005069589033879172</v>
+      </c>
+      <c r="BR58" t="n">
+        <v>0.5121383624712076</v>
+      </c>
+      <c r="BS58" t="n">
+        <v>0.5036850070458383</v>
+      </c>
+      <c r="BT58" t="n">
+        <v>0.0002344512955888229</v>
+      </c>
+      <c r="BU58" t="n">
+        <v>0.1306934048096201</v>
+      </c>
+      <c r="BV58" t="inlineStr"/>
+      <c r="BW58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_sh_seed77_pre2_roll_lr3e4_pen5_cuda</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>77</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>8</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G59" t="n">
+        <v>100</v>
+      </c>
+      <c r="H59" t="n">
+        <v>100</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.667075343417556</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.2954301757812501</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.3013054061041565</v>
+      </c>
+      <c r="L59" t="n">
+        <v>21</v>
+      </c>
+      <c r="M59" t="n">
+        <v>22.04545454545455</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0</v>
+      </c>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="n">
+        <v>40.48681777156889</v>
+      </c>
+      <c r="S59" t="n">
+        <v>2.010435484087793</v>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U59" t="n">
+        <v>708.0450208187103</v>
+      </c>
+      <c r="V59" t="n">
+        <v>0.667075343417556</v>
+      </c>
+      <c r="W59" t="n">
+        <v>0</v>
+      </c>
+      <c r="X59" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y59" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>0.3693231610733474</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>3.540439432613772e-05</v>
+      </c>
+      <c r="AB59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD59" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE59" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF59" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG59" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH59" t="n">
+        <v>22.66666666666667</v>
+      </c>
+      <c r="AI59" t="n">
+        <v>0.5634361698190111</v>
+      </c>
+      <c r="AJ59" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK59" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR59" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS59" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT59" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU59" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV59" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX59" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA59" t="n">
+        <v>-0.0004625957581627461</v>
+      </c>
+      <c r="BB59" t="n">
+        <v>0.006347147537846617</v>
+      </c>
+      <c r="BC59" t="n">
+        <v>0.4536082474226804</v>
+      </c>
+      <c r="BD59" t="n">
+        <v>0.0002571621854530321</v>
+      </c>
+      <c r="BE59" t="n">
+        <v>0.5360824742268041</v>
+      </c>
+      <c r="BF59" t="n">
+        <v>0.3809523809523809</v>
+      </c>
+      <c r="BG59" t="n">
+        <v>0.5431034482758621</v>
+      </c>
+      <c r="BH59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI59" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ59" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK59" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM59" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN59" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO59" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP59" t="n">
+        <v>0.5020865168153625</v>
+      </c>
+      <c r="BQ59" t="n">
+        <v>0.005153197133145535</v>
+      </c>
+      <c r="BR59" t="n">
+        <v>0.5137780584010881</v>
+      </c>
+      <c r="BS59" t="n">
+        <v>0.5067086452675849</v>
+      </c>
+      <c r="BT59" t="n">
+        <v>0.0006009711094858297</v>
+      </c>
+      <c r="BU59" t="n">
+        <v>0.09628777396433132</v>
+      </c>
+      <c r="BV59" t="inlineStr"/>
+      <c r="BW59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_nas100_seed47_pre2_roll_lr3e4_cuda</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>47</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>8</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G60" t="n">
+        <v>100</v>
+      </c>
+      <c r="H60" t="n">
+        <v>100</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.7918185670814138</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.47607080078125</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.2799014429210535</v>
+      </c>
+      <c r="L60" t="n">
+        <v>115</v>
+      </c>
+      <c r="M60" t="n">
+        <v>4.982758620689655</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0</v>
+      </c>
+      <c r="P60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" t="n">
+        <v>94.70746595598757</v>
+      </c>
+      <c r="S60" t="n">
+        <v>5.915379079640843</v>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U60" t="n">
+        <v>721.7437150478363</v>
+      </c>
+      <c r="V60" t="n">
+        <v>-9.208181432918586</v>
+      </c>
+      <c r="W60" t="n">
+        <v>10</v>
+      </c>
+      <c r="X60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>0.1086525399017692</v>
+      </c>
+      <c r="AA60" t="n">
+        <v>5.448362083038763e-05</v>
+      </c>
+      <c r="AB60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD60" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE60" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF60" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG60" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH60" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ60" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK60" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP60" t="n">
+        <v>115</v>
+      </c>
+      <c r="AQ60" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR60" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT60" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU60" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV60" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW60" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX60" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA60" t="n">
+        <v>0.0003151853938843204</v>
+      </c>
+      <c r="BB60" t="n">
+        <v>0.003363679288133212</v>
+      </c>
+      <c r="BC60" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BD60" t="n">
+        <v>-7.247850534531923e-05</v>
+      </c>
+      <c r="BE60" t="n">
+        <v>0.5224913494809689</v>
+      </c>
+      <c r="BF60" t="n">
+        <v>0.5565217391304348</v>
+      </c>
+      <c r="BG60" t="n">
+        <v>0.5140388768898488</v>
+      </c>
+      <c r="BH60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI60" t="n">
+        <v>2</v>
+      </c>
+      <c r="BJ60" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK60" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL60" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM60" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN60" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO60" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP60" t="n">
+        <v>0.5012940040509181</v>
+      </c>
+      <c r="BQ60" t="n">
+        <v>0.00462061487177345</v>
+      </c>
+      <c r="BR60" t="n">
+        <v>0.5118143895196254</v>
+      </c>
+      <c r="BS60" t="n">
+        <v>0.5035790250375609</v>
+      </c>
+      <c r="BT60" t="n">
+        <v>2.99678843736908e-05</v>
+      </c>
+      <c r="BU60" t="n">
+        <v>0.1305825604080741</v>
+      </c>
+      <c r="BV60" t="inlineStr"/>
+      <c r="BW60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_sh_seed77_rtg_lr3e4_pen5_cuda</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>77</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G61" t="n">
+        <v>100</v>
+      </c>
+      <c r="H61" t="n">
+        <v>100</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.7470146886100367</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.3444512939453126</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.2350749257725366</v>
+      </c>
+      <c r="L61" t="n">
+        <v>20</v>
+      </c>
+      <c r="M61" t="n">
+        <v>23.09523809523809</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0</v>
+      </c>
+      <c r="P61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="n">
+        <v>39.85161490179598</v>
+      </c>
+      <c r="S61" t="n">
+        <v>2.092314524867106</v>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U61" t="n">
+        <v>624.5953636169434</v>
+      </c>
+      <c r="V61" t="n">
+        <v>0.7470146886100367</v>
+      </c>
+      <c r="W61" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y61" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z61" t="n">
+        <v>0.3704899165630083</v>
+      </c>
+      <c r="AA61" t="n">
+        <v>3.453995185041362e-05</v>
+      </c>
+      <c r="AB61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD61" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE61" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF61" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG61" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH61" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="AI61" t="n">
+        <v>0.7664854858377946</v>
+      </c>
+      <c r="AJ61" t="n">
+        <v>22</v>
+      </c>
+      <c r="AK61" t="n">
+        <v>24</v>
+      </c>
+      <c r="AL61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR61" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS61" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT61" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU61" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV61" t="inlineStr">
+        <is>
+          <t>reward_to_go</t>
+        </is>
+      </c>
+      <c r="AW61" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AX61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA61" t="n">
+        <v>-0.0003990334039193952</v>
+      </c>
+      <c r="BB61" t="n">
+        <v>0.006323365464424907</v>
+      </c>
+      <c r="BC61" t="n">
+        <v>0.4536082474226804</v>
+      </c>
+      <c r="BD61" t="n">
+        <v>0.0004635664839033498</v>
+      </c>
+      <c r="BE61" t="n">
+        <v>0.5381443298969072</v>
+      </c>
+      <c r="BF61" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BG61" t="n">
+        <v>0.5440860215053763</v>
+      </c>
+      <c r="BH61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ61" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK61" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL61" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM61" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN61" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO61" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP61" t="n">
+        <v>0.5030037485447126</v>
+      </c>
+      <c r="BQ61" t="n">
+        <v>0.005188937687804711</v>
+      </c>
+      <c r="BR61" t="n">
+        <v>0.5146657019546351</v>
+      </c>
+      <c r="BS61" t="n">
+        <v>0.5076600222243476</v>
+      </c>
+      <c r="BT61" t="n">
+        <v>0.0006230517544966076</v>
+      </c>
+      <c r="BU61" t="n">
+        <v>0.09627983405725243</v>
+      </c>
+      <c r="BV61" t="inlineStr"/>
+      <c r="BW61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_nas100_seed47_rtg_lr3e4_cuda</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>47</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>8</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G62" t="n">
+        <v>100</v>
+      </c>
+      <c r="H62" t="n">
+        <v>100</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.7918185670814138</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.47607080078125</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.2799014429210535</v>
+      </c>
+      <c r="L62" t="n">
+        <v>115</v>
+      </c>
+      <c r="M62" t="n">
+        <v>4.982758620689655</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="n">
+        <v>94.70746595598757</v>
+      </c>
+      <c r="S62" t="n">
+        <v>5.915379079640843</v>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U62" t="n">
+        <v>632.9459798336029</v>
+      </c>
+      <c r="V62" t="n">
+        <v>-9.208181432918586</v>
+      </c>
+      <c r="W62" t="n">
+        <v>10</v>
+      </c>
+      <c r="X62" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z62" t="n">
+        <v>0.1110760246734748</v>
+      </c>
+      <c r="AA62" t="n">
+        <v>5.72262439599837e-05</v>
+      </c>
+      <c r="AB62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD62" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE62" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF62" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP62" t="n">
+        <v>115</v>
+      </c>
+      <c r="AQ62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR62" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS62" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT62" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU62" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV62" t="inlineStr">
+        <is>
+          <t>reward_to_go</t>
+        </is>
+      </c>
+      <c r="AW62" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AX62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA62" t="n">
+        <v>0.0003151853938843204</v>
+      </c>
+      <c r="BB62" t="n">
+        <v>0.003363679288133212</v>
+      </c>
+      <c r="BC62" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BD62" t="n">
+        <v>-7.247850534531923e-05</v>
+      </c>
+      <c r="BE62" t="n">
+        <v>0.5224913494809689</v>
+      </c>
+      <c r="BF62" t="n">
+        <v>0.5565217391304348</v>
+      </c>
+      <c r="BG62" t="n">
+        <v>0.5140388768898488</v>
+      </c>
+      <c r="BH62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ62" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK62" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL62" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM62" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN62" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO62" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP62" t="n">
+        <v>0.5015895465666035</v>
+      </c>
+      <c r="BQ62" t="n">
+        <v>0.004619030576640584</v>
+      </c>
+      <c r="BR62" t="n">
+        <v>0.5120124391515363</v>
+      </c>
+      <c r="BS62" t="n">
+        <v>0.5039000160038265</v>
+      </c>
+      <c r="BT62" t="n">
+        <v>1.839781643268507e-05</v>
+      </c>
+      <c r="BU62" t="n">
+        <v>0.1305730907716966</v>
+      </c>
+      <c r="BV62" t="inlineStr"/>
+      <c r="BW62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_sh_seed77_holdbias025_maskage_cuda</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>77</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>8</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G63" t="n">
+        <v>100</v>
+      </c>
+      <c r="H63" t="n">
+        <v>100</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0.4880664263168842</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.1888701171875</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.2909074889806111</v>
+      </c>
+      <c r="L63" t="n">
+        <v>16</v>
+      </c>
+      <c r="M63" t="n">
+        <v>28.52941176470588</v>
+      </c>
+      <c r="N63" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0</v>
+      </c>
+      <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" t="n">
+        <v>35.90902973338962</v>
+      </c>
+      <c r="S63" t="n">
+        <v>1.708368618245004</v>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U63" t="n">
+        <v>611.4529845714569</v>
+      </c>
+      <c r="V63" t="n">
+        <v>-4.511933573683116</v>
+      </c>
+      <c r="W63" t="n">
+        <v>5</v>
+      </c>
+      <c r="X63" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y63" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z63" t="n">
+        <v>0.3554082868038414</v>
+      </c>
+      <c r="AA63" t="n">
+        <v>2.77144412446406e-05</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD63" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE63" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF63" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG63" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH63" t="n">
+        <v>29</v>
+      </c>
+      <c r="AI63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ63" t="n">
+        <v>29</v>
+      </c>
+      <c r="AK63" t="n">
+        <v>29</v>
+      </c>
+      <c r="AL63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN63" t="n">
+        <v>16</v>
+      </c>
+      <c r="AO63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR63" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS63" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT63" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU63" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV63" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA63" t="n">
+        <v>-0.0001829020597086259</v>
+      </c>
+      <c r="BB63" t="n">
+        <v>0.006224662705220176</v>
+      </c>
+      <c r="BC63" t="n">
+        <v>0.4494845360824742</v>
+      </c>
+      <c r="BD63" t="n">
+        <v>0.0001569713028711891</v>
+      </c>
+      <c r="BE63" t="n">
+        <v>0.554639175257732</v>
+      </c>
+      <c r="BF63" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="BG63" t="n">
+        <v>0.5543710021321961</v>
+      </c>
+      <c r="BH63" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK63" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL63" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM63" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN63" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO63" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP63" t="n">
+        <v>0.5015288231913576</v>
+      </c>
+      <c r="BQ63" t="n">
+        <v>0.005224052995212914</v>
+      </c>
+      <c r="BR63" t="n">
+        <v>0.5127347180523824</v>
+      </c>
+      <c r="BS63" t="n">
+        <v>0.5064236030750668</v>
+      </c>
+      <c r="BT63" t="n">
+        <v>0.0006063440500172911</v>
+      </c>
+      <c r="BU63" t="n">
+        <v>0.09622480197972857</v>
+      </c>
+      <c r="BV63" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BW63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_nas100_seed47_holdbias025_maskage_cuda</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>47</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>8</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G64" t="n">
+        <v>100</v>
+      </c>
+      <c r="H64" t="n">
+        <v>100</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0.8906896749616092</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.6065552978515625</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.3134227093162201</v>
+      </c>
+      <c r="L64" t="n">
+        <v>9</v>
+      </c>
+      <c r="M64" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="N64" t="n">
+        <v>0</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" t="n">
+        <v>22.84844140894711</v>
+      </c>
+      <c r="S64" t="n">
+        <v>1.494537926948396</v>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U64" t="n">
+        <v>630.9794900417328</v>
+      </c>
+      <c r="V64" t="n">
+        <v>-9.109310325038392</v>
+      </c>
+      <c r="W64" t="n">
+        <v>10</v>
+      </c>
+      <c r="X64" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y64" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z64" t="n">
+        <v>0.3843804936651461</v>
+      </c>
+      <c r="AA64" t="n">
+        <v>2.721103098848267e-05</v>
+      </c>
+      <c r="AB64" t="n">
+        <v>0.9999242358737521</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>7.575252837139285e-05</v>
+      </c>
+      <c r="AD64" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE64" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF64" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG64" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH64" t="n">
+        <v>60</v>
+      </c>
+      <c r="AI64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ64" t="n">
+        <v>60</v>
+      </c>
+      <c r="AK64" t="n">
+        <v>60</v>
+      </c>
+      <c r="AL64" t="n">
+        <v>9</v>
+      </c>
+      <c r="AM64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN64" t="n">
+        <v>9</v>
+      </c>
+      <c r="AO64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR64" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS64" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT64" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU64" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV64" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA64" t="n">
+        <v>2.45713449170278e-05</v>
+      </c>
+      <c r="BB64" t="n">
+        <v>0.004036170256865504</v>
+      </c>
+      <c r="BC64" t="n">
+        <v>0.4809688581314879</v>
+      </c>
+      <c r="BD64" t="n">
+        <v>-3.70032686553251e-05</v>
+      </c>
+      <c r="BE64" t="n">
+        <v>0.5173010380622838</v>
+      </c>
+      <c r="BF64" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="BG64" t="n">
+        <v>0.5184534270650264</v>
+      </c>
+      <c r="BH64" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK64" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL64" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM64" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN64" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO64" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP64" t="n">
+        <v>0.5027285938031946</v>
+      </c>
+      <c r="BQ64" t="n">
+        <v>0.004990242486078434</v>
+      </c>
+      <c r="BR64" t="n">
+        <v>0.512211351555524</v>
+      </c>
+      <c r="BS64" t="n">
+        <v>0.5055886016172522</v>
+      </c>
+      <c r="BT64" t="n">
+        <v>0.000381304232313404</v>
+      </c>
+      <c r="BU64" t="n">
+        <v>0.1304533070140231</v>
+      </c>
+      <c r="BV64" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BW64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_sh_seed77_holdbias005_late65_cuda</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>77</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>8</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G65" t="n">
+        <v>100</v>
+      </c>
+      <c r="H65" t="n">
+        <v>100</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.1779997413039282</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.02676037597656244</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.3513476666547557</v>
+      </c>
+      <c r="L65" t="n">
+        <v>24</v>
+      </c>
+      <c r="M65" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="n">
+        <v>44.87398247048259</v>
+      </c>
+      <c r="S65" t="n">
+        <v>1.990895594441099</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U65" t="n">
+        <v>616.5501136779785</v>
+      </c>
+      <c r="V65" t="n">
+        <v>0.1779997413039282</v>
+      </c>
+      <c r="W65" t="n">
+        <v>0</v>
+      </c>
+      <c r="X65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y65" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z65" t="n">
+        <v>0.3778054931179588</v>
+      </c>
+      <c r="AA65" t="n">
+        <v>4.072593748949856e-05</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD65" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE65" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF65" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG65" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH65" t="n">
+        <v>20</v>
+      </c>
+      <c r="AI65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ65" t="n">
+        <v>20</v>
+      </c>
+      <c r="AK65" t="n">
+        <v>20</v>
+      </c>
+      <c r="AL65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR65" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT65" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU65" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV65" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW65" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA65" t="n">
+        <v>-1.610528087224235e-06</v>
+      </c>
+      <c r="BB65" t="n">
+        <v>0.006609389884997466</v>
+      </c>
+      <c r="BC65" t="n">
+        <v>0.5030927835051546</v>
+      </c>
+      <c r="BD65" t="n">
+        <v>-0.0001407318982564527</v>
+      </c>
+      <c r="BE65" t="n">
+        <v>0.4804123711340206</v>
+      </c>
+      <c r="BF65" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="BG65" t="n">
+        <v>0.4880694143167028</v>
+      </c>
+      <c r="BH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK65" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL65" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN65" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO65" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP65" t="n">
+        <v>0.5014573945827091</v>
+      </c>
+      <c r="BQ65" t="n">
+        <v>0.005201950298199795</v>
+      </c>
+      <c r="BR65" t="n">
+        <v>0.5126328548205268</v>
+      </c>
+      <c r="BS65" t="n">
+        <v>0.5062467951135537</v>
+      </c>
+      <c r="BT65" t="n">
+        <v>0.0005670976664237294</v>
+      </c>
+      <c r="BU65" t="n">
+        <v>0.09623805462699575</v>
+      </c>
+      <c r="BV65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BW65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>pg_full_gate_holddelta_nas100_seed47_holdbias005_late65_cuda</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>47</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>8</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G66" t="n">
+        <v>100</v>
+      </c>
+      <c r="H66" t="n">
+        <v>100</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.696619445281449</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.3858731689453125</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.2957008053600412</v>
+      </c>
+      <c r="L66" t="n">
+        <v>14</v>
+      </c>
+      <c r="M66" t="n">
+        <v>38.53333333333333</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="n">
+        <v>26.42266099154949</v>
+      </c>
+      <c r="S66" t="n">
+        <v>1.61385272705229</v>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U66" t="n">
+        <v>643.795615196228</v>
+      </c>
+      <c r="V66" t="n">
+        <v>0.696619445281449</v>
+      </c>
+      <c r="W66" t="n">
+        <v>0</v>
+      </c>
+      <c r="X66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y66" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z66" t="n">
+        <v>0.4247167269776139</v>
+      </c>
+      <c r="AA66" t="n">
+        <v>4.059424888206801e-05</v>
+      </c>
+      <c r="AB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD66" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE66" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF66" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG66" t="n">
+        <v>5</v>
+      </c>
+      <c r="AH66" t="n">
+        <v>41</v>
+      </c>
+      <c r="AI66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ66" t="n">
+        <v>41</v>
+      </c>
+      <c r="AK66" t="n">
+        <v>41</v>
+      </c>
+      <c r="AL66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR66" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="AS66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT66" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU66" t="n">
+        <v>5</v>
+      </c>
+      <c r="AV66" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW66" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA66" t="n">
+        <v>0.0002587491067957816</v>
+      </c>
+      <c r="BB66" t="n">
+        <v>0.003839391251263824</v>
+      </c>
+      <c r="BC66" t="n">
+        <v>0.4896193771626298</v>
+      </c>
+      <c r="BD66" t="n">
+        <v>-0.0002461872313326309</v>
+      </c>
+      <c r="BE66" t="n">
+        <v>0.5103806228373703</v>
+      </c>
+      <c r="BF66" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BG66" t="n">
+        <v>0.5106382978723404</v>
+      </c>
+      <c r="BH66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ66" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK66" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL66" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM66" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN66" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO66" t="inlineStr">
+        <is>
+          <t>hold_delta</t>
+        </is>
+      </c>
+      <c r="BP66" t="n">
+        <v>0.5026352226631039</v>
+      </c>
+      <c r="BQ66" t="n">
+        <v>0.005042917985686827</v>
+      </c>
+      <c r="BR66" t="n">
+        <v>0.5123308988797211</v>
+      </c>
+      <c r="BS66" t="n">
+        <v>0.5055789761889765</v>
+      </c>
+      <c r="BT66" t="n">
+        <v>0.000200749971353204</v>
+      </c>
+      <c r="BU66" t="n">
+        <v>0.1304971104210636</v>
+      </c>
+      <c r="BV66" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BW66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pg_full_gate_full_sh_seed77_oldcfg_near2_cuda</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>77</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G67" t="n">
+        <v>100</v>
+      </c>
+      <c r="H67" t="n">
+        <v>100</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.7795309919648515</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.3557951660156251</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.1899508404349509</v>
+      </c>
+      <c r="L67" t="n">
+        <v>22</v>
+      </c>
+      <c r="M67" t="n">
+        <v>21.08695652173913</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" t="n">
+        <v>43.47014394588768</v>
+      </c>
+      <c r="S67" t="n">
+        <v>2.296238630224252</v>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U67" t="n">
+        <v>621.7587914466858</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0.7795309919648515</v>
+      </c>
+      <c r="W67" t="n">
+        <v>0</v>
+      </c>
+      <c r="X67" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>0.3895502461696562</v>
+      </c>
+      <c r="AA67" t="n">
+        <v>0.01632919239621329</v>
+      </c>
+      <c r="AB67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD67" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE67" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF67" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG67" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH67" t="n">
+        <v>21.27272727272727</v>
+      </c>
+      <c r="AI67" t="n">
+        <v>0.4453617714151233</v>
+      </c>
+      <c r="AJ67" t="n">
+        <v>21</v>
+      </c>
+      <c r="AK67" t="n">
+        <v>22</v>
+      </c>
+      <c r="AL67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR67" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT67" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU67" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV67" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW67" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA67" t="n">
+        <v>-0.0004256105913958253</v>
+      </c>
+      <c r="BB67" t="n">
+        <v>0.006221844219979494</v>
+      </c>
+      <c r="BC67" t="n">
+        <v>0.4762886597938144</v>
+      </c>
+      <c r="BD67" t="n">
+        <v>0.0004248592905945039</v>
+      </c>
+      <c r="BE67" t="n">
+        <v>0.5237113402061856</v>
+      </c>
+      <c r="BF67" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BG67" t="n">
+        <v>0.5248380129589633</v>
+      </c>
+      <c r="BH67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK67" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL67" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM67" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN67" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO67" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP67" t="n">
+        <v>0.5012278853617993</v>
+      </c>
+      <c r="BQ67" t="n">
+        <v>0.005278454494384147</v>
+      </c>
+      <c r="BR67" t="n">
+        <v>0.5134188107608519</v>
+      </c>
+      <c r="BS67" t="n">
+        <v>0.5060324295279905</v>
+      </c>
+      <c r="BT67" t="n">
+        <v>0.0006669321080631356</v>
+      </c>
+      <c r="BU67" t="n">
+        <v>0.09630598319867223</v>
+      </c>
+      <c r="BV67" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>pg_full_gate_full_nas100_seed47_oldcfg_min10_cuda</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>47</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>8</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G68" t="n">
+        <v>100</v>
+      </c>
+      <c r="H68" t="n">
+        <v>100</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.9348643581846986</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.6132845458984375</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.2521218627704563</v>
+      </c>
+      <c r="L68" t="n">
+        <v>15</v>
+      </c>
+      <c r="M68" t="n">
+        <v>36.125</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" t="n">
+        <v>28.37377342954278</v>
+      </c>
+      <c r="S68" t="n">
+        <v>1.791052128013689</v>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U68" t="n">
+        <v>631.0385518074036</v>
+      </c>
+      <c r="V68" t="n">
+        <v>0.9348643581846986</v>
+      </c>
+      <c r="W68" t="n">
+        <v>0</v>
+      </c>
+      <c r="X68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>0.4281295288876215</v>
+      </c>
+      <c r="AA68" t="n">
+        <v>0.01640584099178131</v>
+      </c>
+      <c r="AB68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD68" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE68" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF68" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG68" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH68" t="n">
+        <v>37.06666666666667</v>
+      </c>
+      <c r="AI68" t="n">
+        <v>0.4422166387140533</v>
+      </c>
+      <c r="AJ68" t="n">
+        <v>36</v>
+      </c>
+      <c r="AK68" t="n">
+        <v>38</v>
+      </c>
+      <c r="AL68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR68" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AS68" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT68" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU68" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV68" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX68" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA68" t="n">
+        <v>3.809538748887509e-05</v>
+      </c>
+      <c r="BB68" t="n">
+        <v>0.004118260128590642</v>
+      </c>
+      <c r="BC68" t="n">
+        <v>0.4757785467128028</v>
+      </c>
+      <c r="BD68" t="n">
+        <v>2.867588238372906e-05</v>
+      </c>
+      <c r="BE68" t="n">
+        <v>0.5259515570934256</v>
+      </c>
+      <c r="BF68" t="n">
+        <v>0.5333333333333333</v>
+      </c>
+      <c r="BG68" t="n">
+        <v>0.5257548845470693</v>
+      </c>
+      <c r="BH68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK68" t="n">
+        <v>10</v>
+      </c>
+      <c r="BL68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM68" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN68" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO68" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP68" t="n">
+        <v>0.501772646260509</v>
+      </c>
+      <c r="BQ68" t="n">
+        <v>0.005111226358831212</v>
+      </c>
+      <c r="BR68" t="n">
+        <v>0.5121553203020128</v>
+      </c>
+      <c r="BS68" t="n">
+        <v>0.5047637342272333</v>
+      </c>
+      <c r="BT68" t="n">
+        <v>3.129620579148684e-05</v>
+      </c>
+      <c r="BU68" t="n">
+        <v>0.1305956409464245</v>
+      </c>
+      <c r="BV68" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW68" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record final risk embedding PG controller results
</commit_message>
<xml_diff>
--- a/result.xlsx
+++ b/result.xlsx
@@ -2364,7 +2364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ6"/>
+  <dimension ref="A1:AW11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2546,6 +2546,71 @@
       <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>avg_p_hold_post_max</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_mean</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_abs_mean</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>cf_switch_advantage_positive_rate</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>chosen_cf_advantage_mean</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>decision_cf_alignment_rate</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>switch_positive_advantage_rate</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>hold_negative_advantage_rate</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>gate_mean</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>gate_std</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>gate_max</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>gate_live</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>gate_switch_minus_hold</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>gate_top5_mass</t>
         </is>
       </c>
     </row>
@@ -2626,6 +2691,19 @@
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2704,6 +2782,19 @@
       <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr"/>
       <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2782,6 +2873,19 @@
       <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2860,6 +2964,19 @@
       <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2967,6 +3084,754 @@
       </c>
       <c r="AJ6" t="n">
         <v>0</v>
+      </c>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr"/>
+      <c r="AQ6" t="inlineStr"/>
+      <c r="AR6" t="inlineStr"/>
+      <c r="AS6" t="inlineStr"/>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>risk_lite_smoke_nas100</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.2733050537109376</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.7008060046297808</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2166235510805638</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3.235132878132062</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.06201054107715998</v>
+      </c>
+      <c r="I7" t="n">
+        <v>11.30139939826958</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1273.305053710938</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>89</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.929978780448437</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.1105273537687026</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>29</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.3258426966292135</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0.005975022771094649</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>5.977502041787375e-06</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0.01755637399338443</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0.9824436224740127</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>-0.0007068196794258829</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0.00781030654501735</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0.449438202247191</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0.0007068196794258829</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0.550561797752809</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0.550561797752809</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0.5077893633521005</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0.005769312509932042</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0.5197234260901976</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0.5078428508190627</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.00276320670427901</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.130471752935581</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>risk_lite_full_nas100_ep20_mb5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1.91310009765625</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.2202514333258723</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2162570066007881</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.0184706919011</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3067952053260513</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.7179102617092535</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2913.10009765625</v>
+      </c>
+      <c r="K8" t="n">
+        <v>147</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9.243243243243244</v>
+      </c>
+      <c r="M8" t="n">
+        <v>163.1039097439498</v>
+      </c>
+      <c r="N8" t="n">
+        <v>15.74833743082127</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>9.278911564625851</v>
+      </c>
+      <c r="T8" t="n">
+        <v>8.257573158111706</v>
+      </c>
+      <c r="U8" t="n">
+        <v>5</v>
+      </c>
+      <c r="V8" t="n">
+        <v>44</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>83</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.564625850340136</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0.283190182549062</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0.01880244440650819</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>4.116160638850966e-05</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0.003861841079009675</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0.4985380116959064</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>-0.0001130629586936138</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0.5036549707602339</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0.5102040816326531</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0.5028665028665029</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0.501692873627296</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0.009402231590370293</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0.5231393880227155</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>0.5033121114672973</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>-0.0006683387442610065</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.1321939571776934</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>risk_lite_full_sh_ep20_mb5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.7407202148437499</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.1385745395739459</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.2305264258133365</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.6011221189666659</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.2925072800882317</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.473747302271155</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1740.72021484375</v>
+      </c>
+      <c r="K9" t="n">
+        <v>107</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11.53703703703704</v>
+      </c>
+      <c r="M9" t="n">
+        <v>169.1025584358722</v>
+      </c>
+      <c r="N9" t="n">
+        <v>11.90278295826283</v>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="n">
+        <v>11.55140186915888</v>
+      </c>
+      <c r="T9" t="n">
+        <v>7.210109264418697</v>
+      </c>
+      <c r="U9" t="n">
+        <v>5</v>
+      </c>
+      <c r="V9" t="n">
+        <v>23</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>41</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.3831775700934579</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>0.3089277379178886</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0.01765381081963246</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>-0.0002858415796319815</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0.007268302047273509</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0.471107544141252</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.0001277834320714455</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0.5264847512038523</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0.485981308411215</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0.5302897278314311</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0.508885010646396</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0.0105115824541971</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.5326829016399995</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>0.5168546038062385</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.001181987252096772</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.09786835724239748</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pg_risk_final_v1_ep20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2.395419921875</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2483149286154218</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.2156572867871302</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.151433001873</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2932507596088388</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.846766502767048</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3395.419921875</v>
+      </c>
+      <c r="K10" t="n">
+        <v>254</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5.364705882352941</v>
+      </c>
+      <c r="M10" t="n">
+        <v>233.1859735399485</v>
+      </c>
+      <c r="N10" t="n">
+        <v>27.40043894972769</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="n">
+        <v>5.377952755905512</v>
+      </c>
+      <c r="T10" t="n">
+        <v>3.346002748275735</v>
+      </c>
+      <c r="U10" t="n">
+        <v>5</v>
+      </c>
+      <c r="V10" t="n">
+        <v>55</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0.003937007874015748</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>244</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.9606299212598425</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>0.1336161849527684</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>5.242362556436323e-05</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>-4.823624697016986e-05</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0.003763138587619749</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0.5021929824561403</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>7.446972891259533e-05</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0.5095029239766082</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0.531496062992126</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0.5044883303411131</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0.5013129179371379</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0.02327987941986832</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.5428368282335544</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>0.5083485070986358</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>9.019542048067094e-05</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.137048357694644</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pg_risk_final_v1_ep20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pg_controller</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5058793945312501</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.1097196654214873</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.2322165099549118</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.4724886301921628</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3461621971884871</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.3169602664387461</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1505.87939453125</v>
+      </c>
+      <c r="K11" t="n">
+        <v>41</v>
+      </c>
+      <c r="L11" t="n">
+        <v>29.66666666666667</v>
+      </c>
+      <c r="M11" t="n">
+        <v>91.50264619849622</v>
+      </c>
+      <c r="N11" t="n">
+        <v>6.14116520943935</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>30</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>30</v>
+      </c>
+      <c r="V11" t="n">
+        <v>30</v>
+      </c>
+      <c r="W11" t="n">
+        <v>41</v>
+      </c>
+      <c r="X11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>41</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>0.3604117088588622</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>2.877906722756455e-05</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0.9999303788673587</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>6.961300548537997e-05</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>-0.000143531916731162</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0.008022864517888199</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0.4887640449438202</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>7.323332554946637e-05</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0.507223113964687</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>0.4390243902439024</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>0.5095435684647303</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0.5096033115304683</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0.02199884627184817</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.5485766718992261</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>0.5149979839642588</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>-0.0001411136647314132</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.1004170231210191</v>
       </c>
     </row>
   </sheetData>
@@ -2980,7 +3845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW68"/>
+  <dimension ref="A1:BW75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15963,6 +16828,1679 @@
         <v>0</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>risk_lite_smoke_nas100</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>47</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G69" t="n">
+        <v>100</v>
+      </c>
+      <c r="H69" t="n">
+        <v>100</v>
+      </c>
+      <c r="I69" t="n">
+        <v>3.104039241616181</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.2657496337890626</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.06976561426515504</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" t="n">
+        <v>122</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" t="n">
+        <v>62</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="R69" t="n">
+        <v>2.402610875666142</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0.1423786877421662</v>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U69" t="n">
+        <v>25.45749950408936</v>
+      </c>
+      <c r="V69" t="n">
+        <v>-6196.895960758384</v>
+      </c>
+      <c r="W69" t="n">
+        <v>6200</v>
+      </c>
+      <c r="X69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>0.009532937118931797</v>
+      </c>
+      <c r="AA69" t="n">
+        <v>6.131768350314814e-06</v>
+      </c>
+      <c r="AB69" t="n">
+        <v>0.01837042689083084</v>
+      </c>
+      <c r="AC69" t="n">
+        <v>0.9816295725684012</v>
+      </c>
+      <c r="AD69" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE69" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF69" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR69" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT69" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV69" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW69" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA69" t="n">
+        <v>-6.559457518155571e-05</v>
+      </c>
+      <c r="BB69" t="n">
+        <v>0.003348208966286382</v>
+      </c>
+      <c r="BC69" t="n">
+        <v>0.459016393442623</v>
+      </c>
+      <c r="BD69" t="n">
+        <v>6.559457518155571e-05</v>
+      </c>
+      <c r="BE69" t="n">
+        <v>0.5409836065573771</v>
+      </c>
+      <c r="BF69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG69" t="n">
+        <v>0.5409836065573771</v>
+      </c>
+      <c r="BH69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ69" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK69" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BL69" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM69" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN69" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO69" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP69" t="n">
+        <v>0.5067263218711634</v>
+      </c>
+      <c r="BQ69" t="n">
+        <v>0.006920814258428138</v>
+      </c>
+      <c r="BR69" t="n">
+        <v>0.5206848803113718</v>
+      </c>
+      <c r="BS69" t="n">
+        <v>0.5067522750526178</v>
+      </c>
+      <c r="BT69" t="n">
+        <v>0.004242583712349172</v>
+      </c>
+      <c r="BU69" t="n">
+        <v>0.1308423020556325</v>
+      </c>
+      <c r="BV69" t="n">
+        <v>4</v>
+      </c>
+      <c r="BW69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>risk_lite_smoke_nas100_nohb</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>47</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G70" t="n">
+        <v>100</v>
+      </c>
+      <c r="H70" t="n">
+        <v>100</v>
+      </c>
+      <c r="I70" t="n">
+        <v>2.891177551213474</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.2937257080078124</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.108044585095201</v>
+      </c>
+      <c r="L70" t="n">
+        <v>24</v>
+      </c>
+      <c r="M70" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" t="n">
+        <v>22.29473907873034</v>
+      </c>
+      <c r="S70" t="n">
+        <v>1.318879021331668</v>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U70" t="n">
+        <v>23.50061583518982</v>
+      </c>
+      <c r="V70" t="n">
+        <v>2.391177551213474</v>
+      </c>
+      <c r="W70" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="X70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y70" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z70" t="n">
+        <v>0.1367211207350502</v>
+      </c>
+      <c r="AA70" t="n">
+        <v>0.02553551566159847</v>
+      </c>
+      <c r="AB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD70" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE70" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF70" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG70" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH70" t="n">
+        <v>5</v>
+      </c>
+      <c r="AI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ70" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK70" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP70" t="n">
+        <v>24</v>
+      </c>
+      <c r="AQ70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR70" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT70" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU70" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV70" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW70" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA70" t="n">
+        <v>-0.0002297294789163747</v>
+      </c>
+      <c r="BB70" t="n">
+        <v>0.00307614966970773</v>
+      </c>
+      <c r="BC70" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BD70" t="n">
+        <v>1.93909820423034e-05</v>
+      </c>
+      <c r="BE70" t="n">
+        <v>0.5081967213114754</v>
+      </c>
+      <c r="BF70" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="BG70" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK70" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BL70" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM70" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN70" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO70" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP70" t="n">
+        <v>0.504649923473108</v>
+      </c>
+      <c r="BQ70" t="n">
+        <v>0.007730650471248587</v>
+      </c>
+      <c r="BR70" t="n">
+        <v>0.522552096941432</v>
+      </c>
+      <c r="BS70" t="n">
+        <v>0.5066134946756675</v>
+      </c>
+      <c r="BT70" t="n">
+        <v>0.0003593087284138701</v>
+      </c>
+      <c r="BU70" t="n">
+        <v>0.1315024629479549</v>
+      </c>
+      <c r="BV70" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>risk_lite_smoke_sh_nohb</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>77</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G71" t="n">
+        <v>100</v>
+      </c>
+      <c r="H71" t="n">
+        <v>100</v>
+      </c>
+      <c r="I71" t="n">
+        <v>2.452621039681776</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.3559792480468751</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.1506180002275824</v>
+      </c>
+      <c r="L71" t="n">
+        <v>12</v>
+      </c>
+      <c r="M71" t="n">
+        <v>8.923076923076923</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" t="n">
+        <v>18.86201875843108</v>
+      </c>
+      <c r="S71" t="n">
+        <v>1.196868467202876</v>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>skipped</t>
+        </is>
+      </c>
+      <c r="U71" t="n">
+        <v>24.33887887001038</v>
+      </c>
+      <c r="V71" t="n">
+        <v>2.244287706348442</v>
+      </c>
+      <c r="W71" t="n">
+        <v>0.2083333333333333</v>
+      </c>
+      <c r="X71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y71" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z71" t="n">
+        <v>0.2795762782434708</v>
+      </c>
+      <c r="AA71" t="n">
+        <v>0.01747657131403684</v>
+      </c>
+      <c r="AB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD71" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE71" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF71" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH71" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="AI71" t="n">
+        <v>5.923118547972287</v>
+      </c>
+      <c r="AJ71" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK71" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP71" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ71" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="AR71" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT71" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV71" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW71" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA71" t="n">
+        <v>-0.0001776978506000135</v>
+      </c>
+      <c r="BB71" t="n">
+        <v>0.006952170144108221</v>
+      </c>
+      <c r="BC71" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BD71" t="n">
+        <v>-0.0008299585094611192</v>
+      </c>
+      <c r="BE71" t="n">
+        <v>0.4655172413793103</v>
+      </c>
+      <c r="BF71" t="n">
+        <v>0.1666666666666667</v>
+      </c>
+      <c r="BG71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BH71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK71" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BL71" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM71" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN71" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO71" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP71" t="n">
+        <v>0.5116049716698712</v>
+      </c>
+      <c r="BQ71" t="n">
+        <v>0.01002383142998763</v>
+      </c>
+      <c r="BR71" t="n">
+        <v>0.5333463087164122</v>
+      </c>
+      <c r="BS71" t="n">
+        <v>0.5175320274870971</v>
+      </c>
+      <c r="BT71" t="n">
+        <v>0.001668902431165093</v>
+      </c>
+      <c r="BU71" t="n">
+        <v>0.09759272840516321</v>
+      </c>
+      <c r="BV71" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>risk_lite_full_nas100_ep20_mb5</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>47</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>20</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G72" t="n">
+        <v>100</v>
+      </c>
+      <c r="H72" t="n">
+        <v>100</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.8701434442608036</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.565885498046875</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.2995823399994123</v>
+      </c>
+      <c r="L72" t="n">
+        <v>60</v>
+      </c>
+      <c r="M72" t="n">
+        <v>9.475409836065573</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0</v>
+      </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0</v>
+      </c>
+      <c r="R72" t="n">
+        <v>66.41235525906086</v>
+      </c>
+      <c r="S72" t="n">
+        <v>4.308016057999339</v>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U72" t="n">
+        <v>1447.080468893051</v>
+      </c>
+      <c r="V72" t="n">
+        <v>-2.21318988907253</v>
+      </c>
+      <c r="W72" t="n">
+        <v>3.083333333333333</v>
+      </c>
+      <c r="X72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y72" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z72" t="n">
+        <v>0.2881847279610364</v>
+      </c>
+      <c r="AA72" t="n">
+        <v>0.0191889683582953</v>
+      </c>
+      <c r="AB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD72" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE72" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF72" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG72" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH72" t="n">
+        <v>9.483333333333333</v>
+      </c>
+      <c r="AI72" t="n">
+        <v>7.798486320363001</v>
+      </c>
+      <c r="AJ72" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK72" t="n">
+        <v>32</v>
+      </c>
+      <c r="AL72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP72" t="n">
+        <v>37</v>
+      </c>
+      <c r="AQ72" t="n">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AR72" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT72" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU72" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV72" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW72" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA72" t="n">
+        <v>9.933933651938416e-05</v>
+      </c>
+      <c r="BB72" t="n">
+        <v>0.003784456150727121</v>
+      </c>
+      <c r="BC72" t="n">
+        <v>0.486159169550173</v>
+      </c>
+      <c r="BD72" t="n">
+        <v>-0.0001123150843630664</v>
+      </c>
+      <c r="BE72" t="n">
+        <v>0.5346020761245674</v>
+      </c>
+      <c r="BF72" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BG72" t="n">
+        <v>0.527027027027027</v>
+      </c>
+      <c r="BH72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK72" t="n">
+        <v>5</v>
+      </c>
+      <c r="BL72" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM72" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN72" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO72" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP72" t="n">
+        <v>0.5015092680301634</v>
+      </c>
+      <c r="BQ72" t="n">
+        <v>0.009043190432519081</v>
+      </c>
+      <c r="BR72" t="n">
+        <v>0.5218790645830359</v>
+      </c>
+      <c r="BS72" t="n">
+        <v>0.5034606656298093</v>
+      </c>
+      <c r="BT72" t="n">
+        <v>-0.000869419095412567</v>
+      </c>
+      <c r="BU72" t="n">
+        <v>0.1320500043333608</v>
+      </c>
+      <c r="BV72" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>risk_lite_full_sh_ep20_mb5</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>77</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>20</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="G73" t="n">
+        <v>100</v>
+      </c>
+      <c r="H73" t="n">
+        <v>100</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0.5649179761263445</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.2318176269531249</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.2977716463584811</v>
+      </c>
+      <c r="L73" t="n">
+        <v>40</v>
+      </c>
+      <c r="M73" t="n">
+        <v>11.82926829268293</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>0</v>
+      </c>
+      <c r="R73" t="n">
+        <v>64.21214552037418</v>
+      </c>
+      <c r="S73" t="n">
+        <v>3.128730604832526</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U73" t="n">
+        <v>1442.647846460342</v>
+      </c>
+      <c r="V73" t="n">
+        <v>-1.560082023873655</v>
+      </c>
+      <c r="W73" t="n">
+        <v>2.125</v>
+      </c>
+      <c r="X73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y73" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z73" t="n">
+        <v>0.3115153202095751</v>
+      </c>
+      <c r="AA73" t="n">
+        <v>0.01752333601154847</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD73" t="n">
+        <v>4</v>
+      </c>
+      <c r="AE73" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF73" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG73" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH73" t="n">
+        <v>12.075</v>
+      </c>
+      <c r="AI73" t="n">
+        <v>7.685660348987587</v>
+      </c>
+      <c r="AJ73" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK73" t="n">
+        <v>23</v>
+      </c>
+      <c r="AL73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP73" t="n">
+        <v>17</v>
+      </c>
+      <c r="AQ73" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="AR73" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AS73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT73" t="n">
+        <v>10</v>
+      </c>
+      <c r="AU73" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV73" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW73" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA73" t="n">
+        <v>-0.0003865291357890117</v>
+      </c>
+      <c r="BB73" t="n">
+        <v>0.006520291401214955</v>
+      </c>
+      <c r="BC73" t="n">
+        <v>0.4783505154639175</v>
+      </c>
+      <c r="BD73" t="n">
+        <v>0.0001938113024021432</v>
+      </c>
+      <c r="BE73" t="n">
+        <v>0.5051546391752577</v>
+      </c>
+      <c r="BF73" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="BG73" t="n">
+        <v>0.5146067415730337</v>
+      </c>
+      <c r="BH73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK73" t="n">
+        <v>5</v>
+      </c>
+      <c r="BL73" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM73" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN73" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO73" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP73" t="n">
+        <v>0.5079022429038569</v>
+      </c>
+      <c r="BQ73" t="n">
+        <v>0.01056981715325689</v>
+      </c>
+      <c r="BR73" t="n">
+        <v>0.5319196504415925</v>
+      </c>
+      <c r="BS73" t="n">
+        <v>0.5150248125041883</v>
+      </c>
+      <c r="BT73" t="n">
+        <v>0.001326220684634406</v>
+      </c>
+      <c r="BU73" t="n">
+        <v>0.09784544340728485</v>
+      </c>
+      <c r="BV73" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>pg_risk_final_v1_ep20</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>nas100</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>47</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>20</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" t="n">
+        <v>1</v>
+      </c>
+      <c r="I74" t="n">
+        <v>1.018549370694969</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.7007926025390625</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.2478229975270475</v>
+      </c>
+      <c r="L74" t="n">
+        <v>105</v>
+      </c>
+      <c r="M74" t="n">
+        <v>5.452830188679245</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0</v>
+      </c>
+      <c r="P74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" t="n">
+        <v>97.20097045041621</v>
+      </c>
+      <c r="S74" t="n">
+        <v>6.434286667063134</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U74" t="n">
+        <v>1449.06109380722</v>
+      </c>
+      <c r="V74" t="n">
+        <v>1.018549370694969</v>
+      </c>
+      <c r="W74" t="n">
+        <v>0</v>
+      </c>
+      <c r="X74" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y74" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z74" t="n">
+        <v>0.1398269361840516</v>
+      </c>
+      <c r="AA74" t="n">
+        <v>5.199190922152092e-05</v>
+      </c>
+      <c r="AB74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD74" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE74" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF74" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG74" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH74" t="n">
+        <v>5.485714285714286</v>
+      </c>
+      <c r="AI74" t="n">
+        <v>3.180638707089193</v>
+      </c>
+      <c r="AJ74" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK74" t="n">
+        <v>31</v>
+      </c>
+      <c r="AL74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP74" t="n">
+        <v>100</v>
+      </c>
+      <c r="AQ74" t="n">
+        <v>0.9523809523809523</v>
+      </c>
+      <c r="AR74" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AS74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU74" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV74" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW74" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA74" t="n">
+        <v>1.356725396800329e-06</v>
+      </c>
+      <c r="BB74" t="n">
+        <v>0.003537438282792744</v>
+      </c>
+      <c r="BC74" t="n">
+        <v>0.5034602076124568</v>
+      </c>
+      <c r="BD74" t="n">
+        <v>7.488080752809261e-05</v>
+      </c>
+      <c r="BE74" t="n">
+        <v>0.4948096885813149</v>
+      </c>
+      <c r="BF74" t="n">
+        <v>0.4952380952380953</v>
+      </c>
+      <c r="BG74" t="n">
+        <v>0.4947145877378435</v>
+      </c>
+      <c r="BH74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL74" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM74" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN74" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO74" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP74" t="n">
+        <v>0.5032692755794855</v>
+      </c>
+      <c r="BQ74" t="n">
+        <v>0.0222420043780897</v>
+      </c>
+      <c r="BR74" t="n">
+        <v>0.5431044048091532</v>
+      </c>
+      <c r="BS74" t="n">
+        <v>0.5096684540122438</v>
+      </c>
+      <c r="BT74" t="n">
+        <v>0.000266134626988183</v>
+      </c>
+      <c r="BU74" t="n">
+        <v>0.1366876209844355</v>
+      </c>
+      <c r="BV74" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>pg_risk_final_v1_ep20</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>77</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>20</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0.6430668749679012</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0.27872802734375</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.2252127098810282</v>
+      </c>
+      <c r="L75" t="n">
+        <v>16</v>
+      </c>
+      <c r="M75" t="n">
+        <v>28.52941176470588</v>
+      </c>
+      <c r="N75" t="n">
+        <v>0</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0</v>
+      </c>
+      <c r="P75" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" t="n">
+        <v>34.32145153172314</v>
+      </c>
+      <c r="S75" t="n">
+        <v>1.760035670333309</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="U75" t="n">
+        <v>1509.53551697731</v>
+      </c>
+      <c r="V75" t="n">
+        <v>-0.3569331250320988</v>
+      </c>
+      <c r="W75" t="n">
+        <v>1</v>
+      </c>
+      <c r="X75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y75" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z75" t="n">
+        <v>0.3550924649569068</v>
+      </c>
+      <c r="AA75" t="n">
+        <v>2.881755769350633e-05</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>0.9999304413795471</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>6.955060689506354e-05</v>
+      </c>
+      <c r="AD75" t="n">
+        <v>10</v>
+      </c>
+      <c r="AE75" t="n">
+        <v>32</v>
+      </c>
+      <c r="AF75" t="n">
+        <v>64</v>
+      </c>
+      <c r="AG75" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH75" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ75" t="n">
+        <v>30</v>
+      </c>
+      <c r="AK75" t="n">
+        <v>30</v>
+      </c>
+      <c r="AL75" t="n">
+        <v>16</v>
+      </c>
+      <c r="AM75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN75" t="n">
+        <v>16</v>
+      </c>
+      <c r="AO75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR75" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AS75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU75" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AV75" t="inlineStr">
+        <is>
+          <t>episode_sharpe</t>
+        </is>
+      </c>
+      <c r="AW75" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA75" t="n">
+        <v>-0.0003225022654490757</v>
+      </c>
+      <c r="BB75" t="n">
+        <v>0.006609890745957526</v>
+      </c>
+      <c r="BC75" t="n">
+        <v>0.4927835051546392</v>
+      </c>
+      <c r="BD75" t="n">
+        <v>0.0003772274693042116</v>
+      </c>
+      <c r="BE75" t="n">
+        <v>0.511340206185567</v>
+      </c>
+      <c r="BF75" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="BG75" t="n">
+        <v>0.5095948827292111</v>
+      </c>
+      <c r="BH75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL75" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM75" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="BN75" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO75" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="BP75" t="n">
+        <v>0.5082717587652895</v>
+      </c>
+      <c r="BQ75" t="n">
+        <v>0.02278127440817885</v>
+      </c>
+      <c r="BR75" t="n">
+        <v>0.5472045969717282</v>
+      </c>
+      <c r="BS75" t="n">
+        <v>0.5128601993482137</v>
+      </c>
+      <c r="BT75" t="n">
+        <v>0.0005669718094592549</v>
+      </c>
+      <c r="BU75" t="n">
+        <v>0.1005249007614618</v>
+      </c>
+      <c r="BV75" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW75" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>